<commit_message>
Add materials folder and documents section, C2C style
- Any sheet with a File/Link/URL column renders as document cards with
  View and Download instead of contact cards
- Office formats open via Microsoft's web viewer; PDFs and images open
  directly; everything offers a download
- materials/ holds the uploaded files, with four sample society PDFs
- Documents sheet in data.xlsx acts as the manifest, so the existing
  admin editor already manages it
- Admin: upload a material straight to materials/ via the GitHub API,
  which also appends the Documents row automatically

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -8,6 +8,7 @@
     <sheet name="Emergency" sheetId="3" r:id="rId3"/>
     <sheet name="Services" sheetId="4" r:id="rId4"/>
     <sheet name="Residents" sheetId="5" r:id="rId5"/>
+    <sheet name="Documents" sheetId="6" r:id="rId6"/>
   </sheets>
 </workbook>
 </file>
@@ -402,10 +403,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B7"/>
-  <cols>
-    <col min="1" max="1" width="17.83203125" customWidth="1"/>
-    <col min="2" max="2" width="32.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -473,13 +470,6 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E6"/>
-  <cols>
-    <col min="1" max="1" width="17.83203125" customWidth="1"/>
-    <col min="2" max="2" width="18.83203125" customWidth="1"/>
-    <col min="3" max="3" width="12.83203125" customWidth="1"/>
-    <col min="4" max="4" width="17.83203125" customWidth="1"/>
-    <col min="5" max="5" width="25.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -593,12 +583,6 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D6"/>
-  <cols>
-    <col min="1" max="1" width="15.83203125" customWidth="1"/>
-    <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="17.83203125" customWidth="1"/>
-    <col min="4" max="4" width="19.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -694,12 +678,6 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D11"/>
-  <cols>
-    <col min="1" max="1" width="19.83203125" customWidth="1"/>
-    <col min="2" max="2" width="15.83203125" customWidth="1"/>
-    <col min="3" max="3" width="17.83203125" customWidth="1"/>
-    <col min="4" max="4" width="24.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -865,14 +843,6 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F16"/>
-  <cols>
-    <col min="1" max="1" width="21.83203125" customWidth="1"/>
-    <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="12.83203125" customWidth="1"/>
-    <col min="4" max="4" width="17.83203125" customWidth="1"/>
-    <col min="5" max="5" width="23.83203125" customWidth="1"/>
-    <col min="6" max="6" width="12.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1199,4 +1169,107 @@
     <ignoredError numberStoredAsText="1" sqref="A1:F16"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E5"/>
+  <cols>
+    <col min="1" max="1" width="34.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="45.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="46.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Title</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Category</v>
+      </c>
+      <c r="C1" t="str">
+        <v>File</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Updated</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Notes</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Society Bye-Laws (2024 revision)</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Governance</v>
+      </c>
+      <c r="C2" t="str">
+        <v>materials/Society_Bye_Laws_2024.pdf</v>
+      </c>
+      <c r="D2" t="str">
+        <v>2024-06-18</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Registered bye-laws currently in force</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>AGM Minutes 2025</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Governance</v>
+      </c>
+      <c r="C3" t="str">
+        <v>materials/AGM_Minutes_2025.pdf</v>
+      </c>
+      <c r="D3" t="str">
+        <v>2025-09-20</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Annual general meeting, 14 September 2025</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Maintenance &amp; Water Circular</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Circulars</v>
+      </c>
+      <c r="C4" t="str">
+        <v>materials/Maintenance_Circular_Aug_2025.pdf</v>
+      </c>
+      <c r="D4" t="str">
+        <v>2025-08-01</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Payment dates and revised water timings</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Flat Transfer Application Form</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Forms</v>
+      </c>
+      <c r="C5" t="str">
+        <v>materials/Flat_Transfer_Form.pdf</v>
+      </c>
+      <c r="D5" t="str">
+        <v>2024-11-02</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Submit to the society office with enclosures</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E5"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add House Help section with visiting charges
New "House Help" sheet listing domestic help and tradespeople with what
they do, their timings and what they charge.

Columns named Charges/Rate/Fee/Price/Cost/Amount are detected as a rate
and rendered as a gold badge beside the phone number, rather than being
folded into the generic detail line — the charge is the reason someone
scans this section.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -7,8 +7,9 @@
     <sheet name="Committee" sheetId="2" r:id="rId2"/>
     <sheet name="Emergency" sheetId="3" r:id="rId3"/>
     <sheet name="Services" sheetId="4" r:id="rId4"/>
-    <sheet name="Residents" sheetId="5" r:id="rId5"/>
-    <sheet name="Documents" sheetId="6" r:id="rId6"/>
+    <sheet name="House Help" sheetId="5" r:id="rId5"/>
+    <sheet name="Residents" sheetId="6" r:id="rId6"/>
+    <sheet name="Documents" sheetId="7" r:id="rId7"/>
   </sheets>
 </workbook>
 </file>
@@ -842,6 +843,245 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F11"/>
+  <cols>
+    <col min="1" max="1" width="15.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="16.83203125" customWidth="1"/>
+    <col min="4" max="4" width="22.83203125" customWidth="1"/>
+    <col min="5" max="5" width="17.83203125" customWidth="1"/>
+    <col min="6" max="6" width="32.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Name</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Role</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Charges</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Timings</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Phone</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Notes</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Sunita Bai</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Maid</v>
+      </c>
+      <c r="C2" t="str">
+        <v>₹50 / visit</v>
+      </c>
+      <c r="D2" t="str">
+        <v>7 AM – 11 AM</v>
+      </c>
+      <c r="E2" t="str">
+        <v>+91 90210 33001</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Sweeping, mopping, utensils</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Lata Devi</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Maid</v>
+      </c>
+      <c r="C3" t="str">
+        <v>₹60 / visit</v>
+      </c>
+      <c r="D3" t="str">
+        <v>6 AM – 10 AM</v>
+      </c>
+      <c r="E3" t="str">
+        <v>+91 90210 33002</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Also does ironing on request</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Ramesh Yadav</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Plumber</v>
+      </c>
+      <c r="C4" t="str">
+        <v>₹100 / visit</v>
+      </c>
+      <c r="D4" t="str">
+        <v>On call, 8 AM – 8 PM</v>
+      </c>
+      <c r="E4" t="str">
+        <v>+91 90210 33003</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Parts charged separately</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Naresh Bhoir</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Electrician</v>
+      </c>
+      <c r="C5" t="str">
+        <v>₹120 / visit</v>
+      </c>
+      <c r="D5" t="str">
+        <v>On call, 9 AM – 8 PM</v>
+      </c>
+      <c r="E5" t="str">
+        <v>+91 90210 33004</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Wiring, fans, MCB</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Kamla Bai</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Cook</v>
+      </c>
+      <c r="C6" t="str">
+        <v>₹2,500 / month</v>
+      </c>
+      <c r="D6" t="str">
+        <v>11 AM – 2 PM</v>
+      </c>
+      <c r="E6" t="str">
+        <v>+91 90210 33005</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Vegetarian, 2 meals a day</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Imran Shaikh</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Car Cleaning</v>
+      </c>
+      <c r="C7" t="str">
+        <v>₹500 / month</v>
+      </c>
+      <c r="D7" t="str">
+        <v>6 AM – 9 AM</v>
+      </c>
+      <c r="E7" t="str">
+        <v>+91 90210 33006</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Daily wash, weekly interior</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Deepak Sawant</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Driver</v>
+      </c>
+      <c r="C8" t="str">
+        <v>₹300 / trip</v>
+      </c>
+      <c r="D8" t="str">
+        <v>By appointment</v>
+      </c>
+      <c r="E8" t="str">
+        <v>+91 90210 33007</v>
+      </c>
+      <c r="F8" t="str">
+        <v>Local trips, own licence</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Anita Kamble</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Baby Sitter</v>
+      </c>
+      <c r="C9" t="str">
+        <v>₹150 / hour</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Flexible</v>
+      </c>
+      <c r="E9" t="str">
+        <v>+91 90210 33008</v>
+      </c>
+      <c r="F9" t="str">
+        <v>Experienced with toddlers</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Salim Ansari</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Carpenter</v>
+      </c>
+      <c r="C10" t="str">
+        <v>₹150 / visit</v>
+      </c>
+      <c r="D10" t="str">
+        <v>On call</v>
+      </c>
+      <c r="E10" t="str">
+        <v>+91 90210 33009</v>
+      </c>
+      <c r="F10" t="str">
+        <v>Furniture repair, fittings</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Ganesh Pawar</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Gardener</v>
+      </c>
+      <c r="C11" t="str">
+        <v>₹80 / visit</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Tue &amp; Sat mornings</v>
+      </c>
+      <c r="E11" t="str">
+        <v>+91 90210 33010</v>
+      </c>
+      <c r="F11" t="str">
+        <v>Balcony plants, terrace garden</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:F11"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F16"/>
   <sheetData>
     <row r="1">
@@ -1171,16 +1411,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E5"/>
-  <cols>
-    <col min="1" max="1" width="34.83203125" customWidth="1"/>
-    <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="45.83203125" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" customWidth="1"/>
-    <col min="5" max="5" width="46.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">

</xml_diff>

<commit_message>
Stop trimming card content; merge Services with House Help
Cards were fixed-height rows with nowrap and ellipsis, which clipped
timings and notes once House Help added real detail. Rebuilt as
content-sized cards: header (avatar, name, role, charge badge), then one
wrapped labelled line per detail, then a footer with the full number and
the tap targets. Sidebar rows wrap too.

Services and House Help are now one "Services & Help" sheet — both are
people you ring, and splitting them meant scanning two places.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -6,10 +6,9 @@
     <sheet name="About" sheetId="1" r:id="rId1"/>
     <sheet name="Committee" sheetId="2" r:id="rId2"/>
     <sheet name="Emergency" sheetId="3" r:id="rId3"/>
-    <sheet name="Services" sheetId="4" r:id="rId4"/>
-    <sheet name="House Help" sheetId="5" r:id="rId5"/>
-    <sheet name="Residents" sheetId="6" r:id="rId6"/>
-    <sheet name="Documents" sheetId="7" r:id="rId7"/>
+    <sheet name="Services &amp; Help" sheetId="4" r:id="rId4"/>
+    <sheet name="Residents" sheetId="5" r:id="rId5"/>
+    <sheet name="Documents" sheetId="6" r:id="rId6"/>
   </sheets>
 </workbook>
 </file>
@@ -678,409 +677,404 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:F19"/>
+  <cols>
+    <col min="1" max="1" width="15.83203125" customWidth="1"/>
+    <col min="2" max="2" width="19.83203125" customWidth="1"/>
+    <col min="3" max="3" width="16.83203125" customWidth="1"/>
+    <col min="4" max="4" width="24.83203125" customWidth="1"/>
+    <col min="5" max="5" width="17.83203125" customWidth="1"/>
+    <col min="6" max="6" width="37.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Service</v>
+        <v>Name</v>
       </c>
       <c r="B1" t="str">
-        <v>Contact</v>
+        <v>Role</v>
       </c>
       <c r="C1" t="str">
+        <v>Charges</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Timings</v>
+      </c>
+      <c r="E1" t="str">
         <v>Phone</v>
       </c>
-      <c r="D1" t="str">
+      <c r="F1" t="str">
         <v>Notes</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
+        <v>Santosh Gupta</v>
+      </c>
+      <c r="B2" t="str">
         <v>Plumber</v>
       </c>
-      <c r="B2" t="str">
-        <v>Santosh Gupta</v>
-      </c>
       <c r="C2" t="str">
+        <v>₹100 / visit</v>
+      </c>
+      <c r="D2" t="str">
+        <v>8 AM – 8 PM, on call</v>
+      </c>
+      <c r="E2" t="str">
         <v>+91 90040 55511</v>
       </c>
-      <c r="D2" t="str">
-        <v>9 AM – 7 PM</v>
+      <c r="F2" t="str">
+        <v>Parts charged separately</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
+        <v>Naresh Bhoir</v>
+      </c>
+      <c r="B3" t="str">
         <v>Electrician</v>
       </c>
-      <c r="B3" t="str">
-        <v>Naresh Bhoir</v>
-      </c>
       <c r="C3" t="str">
+        <v>₹120 / visit</v>
+      </c>
+      <c r="D3" t="str">
+        <v>9 AM – 8 PM, on call</v>
+      </c>
+      <c r="E3" t="str">
         <v>+91 90040 55512</v>
       </c>
-      <c r="D3" t="str">
-        <v>9 AM – 8 PM</v>
+      <c r="F3" t="str">
+        <v>Wiring, fans, MCB</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Lift Technician</v>
+        <v>Salim Ansari</v>
       </c>
       <c r="B4" t="str">
-        <v>Otis Service</v>
+        <v>Carpenter</v>
       </c>
       <c r="C4" t="str">
-        <v>+91 90040 55513</v>
+        <v>₹150 / visit</v>
       </c>
       <c r="D4" t="str">
-        <v>AMC — 4 hr response</v>
+        <v>On call</v>
+      </c>
+      <c r="E4" t="str">
+        <v>+91 90210 33009</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Furniture repair and fittings</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Pest Control</v>
+        <v>Otis Service</v>
       </c>
       <c r="B5" t="str">
-        <v>HiCare</v>
+        <v>Lift Technician</v>
       </c>
       <c r="C5" t="str">
-        <v>+91 90040 55514</v>
+        <v>Society AMC</v>
       </c>
       <c r="D5" t="str">
-        <v>Quarterly, by booking</v>
+        <v>4-hour response</v>
+      </c>
+      <c r="E5" t="str">
+        <v>+91 90040 55513</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Report faults to the manager first</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Housekeeping</v>
+        <v>HiCare</v>
       </c>
       <c r="B6" t="str">
-        <v>Shanti Devi</v>
+        <v>Pest Control</v>
       </c>
       <c r="C6" t="str">
-        <v>+91 90040 55515</v>
+        <v>₹1,200 / flat</v>
       </c>
       <c r="D6" t="str">
-        <v>6 AM – 2 PM</v>
+        <v>By appointment</v>
+      </c>
+      <c r="E6" t="str">
+        <v>+91 90040 55514</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Quarterly society drive is free</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Water Tanker</v>
+        <v>Shanti Devi</v>
       </c>
       <c r="B7" t="str">
-        <v>Jai Bhavani</v>
+        <v>Housekeeping</v>
       </c>
       <c r="C7" t="str">
-        <v>+91 90040 55521</v>
+        <v>Society staff</v>
       </c>
       <c r="D7" t="str">
-        <v>Same-day delivery</v>
+        <v>6 AM – 2 PM</v>
+      </c>
+      <c r="E7" t="str">
+        <v>+91 90040 55515</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Common areas and staircases</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Electricity Board</v>
+        <v>Ganesh Pawar</v>
       </c>
       <c r="B8" t="str">
-        <v>MSEDCL</v>
+        <v>Gardener</v>
       </c>
       <c r="C8" t="str">
-        <v>1912</v>
+        <v>₹80 / visit</v>
       </c>
       <c r="D8" t="str">
-        <v>Outage helpline</v>
+        <v>Tue &amp; Sat mornings</v>
+      </c>
+      <c r="E8" t="str">
+        <v>+91 90210 33010</v>
+      </c>
+      <c r="F8" t="str">
+        <v>Balcony and terrace plants</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Gas Agency</v>
+        <v>Jai Bhavani</v>
       </c>
       <c r="B9" t="str">
-        <v>Mahanagar Gas</v>
+        <v>Water Tanker</v>
       </c>
       <c r="C9" t="str">
-        <v>+91 90040 55522</v>
+        <v>₹900 / tanker</v>
       </c>
       <c r="D9" t="str">
-        <v>Leak: 1800 22 9944</v>
+        <v>Same-day delivery</v>
+      </c>
+      <c r="E9" t="str">
+        <v>+91 90040 55521</v>
+      </c>
+      <c r="F9" t="str">
+        <v>10,000 litre tanker</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Society Manager</v>
+        <v>MSEDCL</v>
       </c>
       <c r="B10" t="str">
-        <v>D. Kamble</v>
+        <v>Electricity Board</v>
       </c>
       <c r="C10" t="str">
-        <v>+91 90040 55531</v>
+        <v/>
       </c>
       <c r="D10" t="str">
-        <v>Mon–Sat, 10 AM – 6 PM</v>
+        <v>24x7 helpline</v>
+      </c>
+      <c r="E10" t="str">
+        <v>1912</v>
+      </c>
+      <c r="F10" t="str">
+        <v>Outages and meter faults</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
+        <v>Mahanagar Gas</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Gas Agency</v>
+      </c>
+      <c r="C11" t="str">
+        <v/>
+      </c>
+      <c r="D11" t="str">
+        <v>24x7 for leaks</v>
+      </c>
+      <c r="E11" t="str">
+        <v>+91 90040 55522</v>
+      </c>
+      <c r="F11" t="str">
+        <v>Leak helpline 1800 22 9944</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>D. Kamble</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Society Manager</v>
+      </c>
+      <c r="C12" t="str">
+        <v/>
+      </c>
+      <c r="D12" t="str">
+        <v>Mon–Sat, 10 AM – 6 PM</v>
+      </c>
+      <c r="E12" t="str">
+        <v>+91 90040 55531</v>
+      </c>
+      <c r="F12" t="str">
+        <v>Maintenance bills, NOCs, complaints</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>S. Rane</v>
+      </c>
+      <c r="B13" t="str">
         <v>Accountant</v>
       </c>
-      <c r="B11" t="str">
-        <v>S. Rane</v>
-      </c>
-      <c r="C11" t="str">
+      <c r="C13" t="str">
+        <v/>
+      </c>
+      <c r="D13" t="str">
+        <v>Tue &amp; Thu, 4 PM – 7 PM</v>
+      </c>
+      <c r="E13" t="str">
         <v>+91 90040 55532</v>
       </c>
-      <c r="D11" t="str">
-        <v>Tue &amp; Thu, 4 PM – 7 PM</v>
+      <c r="F13" t="str">
+        <v>Dues, receipts, statements</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Sunita Bai</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Maid</v>
+      </c>
+      <c r="C14" t="str">
+        <v>₹50 / visit</v>
+      </c>
+      <c r="D14" t="str">
+        <v>7 AM – 11 AM</v>
+      </c>
+      <c r="E14" t="str">
+        <v>+91 90210 33001</v>
+      </c>
+      <c r="F14" t="str">
+        <v>Sweeping, mopping, utensils</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Lata Devi</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Maid</v>
+      </c>
+      <c r="C15" t="str">
+        <v>₹60 / visit</v>
+      </c>
+      <c r="D15" t="str">
+        <v>6 AM – 10 AM</v>
+      </c>
+      <c r="E15" t="str">
+        <v>+91 90210 33002</v>
+      </c>
+      <c r="F15" t="str">
+        <v>Also irons clothes on request</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>Kamla Bai</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Cook</v>
+      </c>
+      <c r="C16" t="str">
+        <v>₹2,500 / month</v>
+      </c>
+      <c r="D16" t="str">
+        <v>11 AM – 2 PM</v>
+      </c>
+      <c r="E16" t="str">
+        <v>+91 90210 33005</v>
+      </c>
+      <c r="F16" t="str">
+        <v>Vegetarian, two meals a day</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Imran Shaikh</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Car Cleaning</v>
+      </c>
+      <c r="C17" t="str">
+        <v>₹500 / month</v>
+      </c>
+      <c r="D17" t="str">
+        <v>6 AM – 9 AM</v>
+      </c>
+      <c r="E17" t="str">
+        <v>+91 90210 33006</v>
+      </c>
+      <c r="F17" t="str">
+        <v>Daily wash, interior weekly</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Deepak Sawant</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Driver</v>
+      </c>
+      <c r="C18" t="str">
+        <v>₹300 / trip</v>
+      </c>
+      <c r="D18" t="str">
+        <v>By appointment</v>
+      </c>
+      <c r="E18" t="str">
+        <v>+91 90210 33007</v>
+      </c>
+      <c r="F18" t="str">
+        <v>Local trips, holds a valid licence</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Anita Kamble</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Baby Sitter</v>
+      </c>
+      <c r="C19" t="str">
+        <v>₹150 / hour</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Flexible</v>
+      </c>
+      <c r="E19" t="str">
+        <v>+91 90210 33008</v>
+      </c>
+      <c r="F19" t="str">
+        <v>Experienced with toddlers</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F19"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F11"/>
-  <cols>
-    <col min="1" max="1" width="15.83203125" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" customWidth="1"/>
-    <col min="3" max="3" width="16.83203125" customWidth="1"/>
-    <col min="4" max="4" width="22.83203125" customWidth="1"/>
-    <col min="5" max="5" width="17.83203125" customWidth="1"/>
-    <col min="6" max="6" width="32.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Name</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Role</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Charges</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Timings</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Phone</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Notes</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Sunita Bai</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Maid</v>
-      </c>
-      <c r="C2" t="str">
-        <v>₹50 / visit</v>
-      </c>
-      <c r="D2" t="str">
-        <v>7 AM – 11 AM</v>
-      </c>
-      <c r="E2" t="str">
-        <v>+91 90210 33001</v>
-      </c>
-      <c r="F2" t="str">
-        <v>Sweeping, mopping, utensils</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Lata Devi</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Maid</v>
-      </c>
-      <c r="C3" t="str">
-        <v>₹60 / visit</v>
-      </c>
-      <c r="D3" t="str">
-        <v>6 AM – 10 AM</v>
-      </c>
-      <c r="E3" t="str">
-        <v>+91 90210 33002</v>
-      </c>
-      <c r="F3" t="str">
-        <v>Also does ironing on request</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Ramesh Yadav</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Plumber</v>
-      </c>
-      <c r="C4" t="str">
-        <v>₹100 / visit</v>
-      </c>
-      <c r="D4" t="str">
-        <v>On call, 8 AM – 8 PM</v>
-      </c>
-      <c r="E4" t="str">
-        <v>+91 90210 33003</v>
-      </c>
-      <c r="F4" t="str">
-        <v>Parts charged separately</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Naresh Bhoir</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Electrician</v>
-      </c>
-      <c r="C5" t="str">
-        <v>₹120 / visit</v>
-      </c>
-      <c r="D5" t="str">
-        <v>On call, 9 AM – 8 PM</v>
-      </c>
-      <c r="E5" t="str">
-        <v>+91 90210 33004</v>
-      </c>
-      <c r="F5" t="str">
-        <v>Wiring, fans, MCB</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>Kamla Bai</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Cook</v>
-      </c>
-      <c r="C6" t="str">
-        <v>₹2,500 / month</v>
-      </c>
-      <c r="D6" t="str">
-        <v>11 AM – 2 PM</v>
-      </c>
-      <c r="E6" t="str">
-        <v>+91 90210 33005</v>
-      </c>
-      <c r="F6" t="str">
-        <v>Vegetarian, 2 meals a day</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>Imran Shaikh</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Car Cleaning</v>
-      </c>
-      <c r="C7" t="str">
-        <v>₹500 / month</v>
-      </c>
-      <c r="D7" t="str">
-        <v>6 AM – 9 AM</v>
-      </c>
-      <c r="E7" t="str">
-        <v>+91 90210 33006</v>
-      </c>
-      <c r="F7" t="str">
-        <v>Daily wash, weekly interior</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>Deepak Sawant</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Driver</v>
-      </c>
-      <c r="C8" t="str">
-        <v>₹300 / trip</v>
-      </c>
-      <c r="D8" t="str">
-        <v>By appointment</v>
-      </c>
-      <c r="E8" t="str">
-        <v>+91 90210 33007</v>
-      </c>
-      <c r="F8" t="str">
-        <v>Local trips, own licence</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>Anita Kamble</v>
-      </c>
-      <c r="B9" t="str">
-        <v>Baby Sitter</v>
-      </c>
-      <c r="C9" t="str">
-        <v>₹150 / hour</v>
-      </c>
-      <c r="D9" t="str">
-        <v>Flexible</v>
-      </c>
-      <c r="E9" t="str">
-        <v>+91 90210 33008</v>
-      </c>
-      <c r="F9" t="str">
-        <v>Experienced with toddlers</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>Salim Ansari</v>
-      </c>
-      <c r="B10" t="str">
-        <v>Carpenter</v>
-      </c>
-      <c r="C10" t="str">
-        <v>₹150 / visit</v>
-      </c>
-      <c r="D10" t="str">
-        <v>On call</v>
-      </c>
-      <c r="E10" t="str">
-        <v>+91 90210 33009</v>
-      </c>
-      <c r="F10" t="str">
-        <v>Furniture repair, fittings</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>Ganesh Pawar</v>
-      </c>
-      <c r="B11" t="str">
-        <v>Gardener</v>
-      </c>
-      <c r="C11" t="str">
-        <v>₹80 / visit</v>
-      </c>
-      <c r="D11" t="str">
-        <v>Tue &amp; Sat mornings</v>
-      </c>
-      <c r="E11" t="str">
-        <v>+91 90210 33010</v>
-      </c>
-      <c r="F11" t="str">
-        <v>Balcony plants, terrace garden</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F11"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F16"/>
   <sheetData>
@@ -1411,7 +1405,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E5"/>
   <sheetData>

</xml_diff>

<commit_message>
Add confidentiality banner and per-section disclaimers
"Confidential Notice" in the About sheet renders a site-wide banner.
"Note: <Section name>" attaches a caveat under that section's heading,
so any section can carry one without a code change.

Ships with a members-only sharing notice, and a disclaimer on Services &
Help stating the contacts are resident-supplied, unverified, and engaged
at the reader's own risk.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -402,7 +402,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B9"/>
+  <cols>
+    <col min="1" max="1" width="24.83203125" customWidth="1"/>
+    <col min="2" max="2" width="80.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -460,9 +464,25 @@
         <v>NBOM/HSG/1284/2009</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Confidential Notice</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Please do not forward this link or share these details with anyone outside the society.</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Note: Services &amp; Help</v>
+      </c>
+      <c r="B9" t="str">
+        <v>These contacts are collected from fellow residents. The society has not verified, screened or endorsed any of them. Please check credentials and agree charges before engaging anyone — you do so at your own risk.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B9"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -678,14 +698,6 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F19"/>
-  <cols>
-    <col min="1" max="1" width="15.83203125" customWidth="1"/>
-    <col min="2" max="2" width="19.83203125" customWidth="1"/>
-    <col min="3" max="3" width="16.83203125" customWidth="1"/>
-    <col min="4" max="4" width="24.83203125" customWidth="1"/>
-    <col min="5" max="5" width="17.83203125" customWidth="1"/>
-    <col min="6" max="6" width="37.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">

</xml_diff>

<commit_message>
Show flat owner details on tenanted residents
Columns prefixed Owner or Landlord are grouped and rendered as a
distinct block on the card, with a tappable number. They are claimed
before the generic rules, so "Owner Phone" does not become a call button
for the tenant and "Owner Address" does not merge into their own
address line.

The block appears only when a row carries owner values, so
owner-occupied flats and other sheets are unaffected. The Apps Script
transform now writes these into the public Residents sheet for tenants;
dates of birth stay in _Private.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -403,10 +403,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B9"/>
-  <cols>
-    <col min="1" max="1" width="24.83203125" customWidth="1"/>
-    <col min="2" max="2" width="80.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1088,7 +1084,18 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:I16"/>
+  <cols>
+    <col min="1" max="1" width="21.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="17.83203125" customWidth="1"/>
+    <col min="5" max="5" width="23.83203125" customWidth="1"/>
+    <col min="6" max="6" width="12.83203125" customWidth="1"/>
+    <col min="7" max="7" width="17.83203125" customWidth="1"/>
+    <col min="8" max="8" width="17.83203125" customWidth="1"/>
+    <col min="9" max="9" width="48.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1109,6 +1116,15 @@
       <c r="F1" t="str">
         <v>Type</v>
       </c>
+      <c r="G1" t="str">
+        <v>Owner Name</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Owner Phone</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Owner Address</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -1129,6 +1145,15 @@
       <c r="F2" t="str">
         <v>Owner</v>
       </c>
+      <c r="G2" t="str">
+        <v/>
+      </c>
+      <c r="H2" t="str">
+        <v/>
+      </c>
+      <c r="I2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -1149,6 +1174,15 @@
       <c r="F3" t="str">
         <v>Owner</v>
       </c>
+      <c r="G3" t="str">
+        <v/>
+      </c>
+      <c r="H3" t="str">
+        <v/>
+      </c>
+      <c r="I3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -1169,6 +1203,15 @@
       <c r="F4" t="str">
         <v>Tenant</v>
       </c>
+      <c r="G4" t="str">
+        <v>Sanjay Kulkarni</v>
+      </c>
+      <c r="H4" t="str">
+        <v>+91 98200 44001</v>
+      </c>
+      <c r="I4" t="str">
+        <v>Flat 9, Sunrise Apartments, Aundh, Pune 411007</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -1189,6 +1232,15 @@
       <c r="F5" t="str">
         <v>Owner</v>
       </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
+      <c r="H5" t="str">
+        <v/>
+      </c>
+      <c r="I5" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -1209,6 +1261,15 @@
       <c r="F6" t="str">
         <v>Owner</v>
       </c>
+      <c r="G6" t="str">
+        <v/>
+      </c>
+      <c r="H6" t="str">
+        <v/>
+      </c>
+      <c r="I6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -1229,6 +1290,15 @@
       <c r="F7" t="str">
         <v>Owner</v>
       </c>
+      <c r="G7" t="str">
+        <v/>
+      </c>
+      <c r="H7" t="str">
+        <v/>
+      </c>
+      <c r="I7" t="str">
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -1249,6 +1319,15 @@
       <c r="F8" t="str">
         <v>Owner</v>
       </c>
+      <c r="G8" t="str">
+        <v/>
+      </c>
+      <c r="H8" t="str">
+        <v/>
+      </c>
+      <c r="I8" t="str">
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -1269,6 +1348,15 @@
       <c r="F9" t="str">
         <v>Tenant</v>
       </c>
+      <c r="G9" t="str">
+        <v>Rajesh Menon</v>
+      </c>
+      <c r="H9" t="str">
+        <v>+91 98200 44002</v>
+      </c>
+      <c r="I9" t="str">
+        <v>B-201, Green Valley Residency (resident owner)</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -1289,6 +1377,15 @@
       <c r="F10" t="str">
         <v>Owner</v>
       </c>
+      <c r="G10" t="str">
+        <v/>
+      </c>
+      <c r="H10" t="str">
+        <v/>
+      </c>
+      <c r="I10" t="str">
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -1309,6 +1406,15 @@
       <c r="F11" t="str">
         <v>Owner</v>
       </c>
+      <c r="G11" t="str">
+        <v/>
+      </c>
+      <c r="H11" t="str">
+        <v/>
+      </c>
+      <c r="I11" t="str">
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -1329,6 +1435,15 @@
       <c r="F12" t="str">
         <v>Owner</v>
       </c>
+      <c r="G12" t="str">
+        <v/>
+      </c>
+      <c r="H12" t="str">
+        <v/>
+      </c>
+      <c r="I12" t="str">
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -1349,6 +1464,15 @@
       <c r="F13" t="str">
         <v>Tenant</v>
       </c>
+      <c r="G13" t="str">
+        <v>Farida Merchant</v>
+      </c>
+      <c r="H13" t="str">
+        <v>+91 98200 44003</v>
+      </c>
+      <c r="I13" t="str">
+        <v>22 Peddar Road, Mumbai 400026</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
@@ -1369,6 +1493,15 @@
       <c r="F14" t="str">
         <v>Owner</v>
       </c>
+      <c r="G14" t="str">
+        <v/>
+      </c>
+      <c r="H14" t="str">
+        <v/>
+      </c>
+      <c r="I14" t="str">
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -1389,6 +1522,15 @@
       <c r="F15" t="str">
         <v>Owner</v>
       </c>
+      <c r="G15" t="str">
+        <v/>
+      </c>
+      <c r="H15" t="str">
+        <v/>
+      </c>
+      <c r="I15" t="str">
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
@@ -1409,10 +1551,19 @@
       <c r="F16" t="str">
         <v>Owner</v>
       </c>
+      <c r="G16" t="str">
+        <v/>
+      </c>
+      <c r="H16" t="str">
+        <v/>
+      </c>
+      <c r="I16" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I16"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update directory data (72 rows)
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -9,6 +9,7 @@
     <sheet name="Services &amp; Help" sheetId="4" r:id="rId4"/>
     <sheet name="Residents" sheetId="5" r:id="rId5"/>
     <sheet name="Documents" sheetId="6" r:id="rId6"/>
+    <sheet name="Services" sheetId="7" r:id="rId7"/>
   </sheets>
 </workbook>
 </file>
@@ -402,10 +403,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B7"/>
   <cols>
-    <col min="1" max="1" width="26.83203125" customWidth="1"/>
-    <col min="2" max="2" width="90.83203125" customWidth="1"/>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -421,7 +422,7 @@
         <v>Society Name</v>
       </c>
       <c r="B2" t="str">
-        <v>Green Valley Residency</v>
+        <v>Laxmi venkatesh Nagar</v>
       </c>
     </row>
     <row r="3">
@@ -429,7 +430,7 @@
         <v>Tagline</v>
       </c>
       <c r="B3" t="str">
-        <v>A Co-operative Housing Society</v>
+        <v>Best Housing Society in Ichalkaranji</v>
       </c>
     </row>
     <row r="4">
@@ -437,7 +438,7 @@
         <v>Address</v>
       </c>
       <c r="B4" t="str">
-        <v>Plot 14, Sector 22, Kharghar</v>
+        <v>Old chandur road</v>
       </c>
     </row>
     <row r="5">
@@ -445,7 +446,7 @@
         <v>City</v>
       </c>
       <c r="B5" t="str">
-        <v>Navi Mumbai</v>
+        <v>ichalkaranji</v>
       </c>
     </row>
     <row r="6">
@@ -453,7 +454,7 @@
         <v>Pincode</v>
       </c>
       <c r="B6" t="str">
-        <v>410210</v>
+        <v>416115</v>
       </c>
     </row>
     <row r="7">
@@ -464,81 +465,9 @@
         <v>NBOM/HSG/1284/2009</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>Confidential Notice</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Please do not forward this link or share these details with anyone outside the society.</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>Note: Services &amp; Help</v>
-      </c>
-      <c r="B9" t="str">
-        <v>These contacts are collected from fellow residents. The society has not verified, screened or endorsed any of them. Please check credentials and agree charges before engaging anyone — you do so at your own risk.</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>Hindi: Committee</v>
-      </c>
-      <c r="B10" t="str">
-        <v>समिति</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>Hindi: Emergency</v>
-      </c>
-      <c r="B11" t="str">
-        <v>आपातकालीन संपर्क</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>Hindi: Services &amp; Help</v>
-      </c>
-      <c r="B12" t="str">
-        <v>सेवाएँ और सहायता</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>Hindi: Residents</v>
-      </c>
-      <c r="B13" t="str">
-        <v>निवासी</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>Hindi: Documents</v>
-      </c>
-      <c r="B14" t="str">
-        <v>दस्तावेज़</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>Confidential HI</v>
-      </c>
-      <c r="B15" t="str">
-        <v>कृपया यह लिंक या विवरण सोसाइटी के बाहर किसी के साथ साझा न करें।</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="str">
-        <v>Note HI: Services &amp; Help</v>
-      </c>
-      <c r="B16" t="str">
-        <v>ये संपर्क अन्य निवासियों द्वारा दिए गए हैं। सोसाइटी ने इनकी जाँच नहीं की है। काम शुरू कराने से पहले कृपया स्वयं पुष्टि करें और शुल्क तय कर लें — जोखिम आपका अपना होगा।</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B7"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -546,6 +475,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E6"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -566,7 +502,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Ramesh Iyer</v>
+        <v/>
       </c>
       <c r="B2" t="str">
         <v>Chairman</v>
@@ -575,15 +511,15 @@
         <v>A-402</v>
       </c>
       <c r="D2" t="str">
-        <v>+91 98200 11223</v>
+        <v/>
       </c>
       <c r="E2" t="str">
-        <v>ramesh.iyer@example.com</v>
+        <v/>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Sunita Deshmukh</v>
+        <v/>
       </c>
       <c r="B3" t="str">
         <v>Hon. Secretary</v>
@@ -592,15 +528,15 @@
         <v>B-105</v>
       </c>
       <c r="D3" t="str">
-        <v>+91 98200 11224</v>
+        <v/>
       </c>
       <c r="E3" t="str">
-        <v>sunita.d@example.com</v>
+        <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Farhan Qureshi</v>
+        <v/>
       </c>
       <c r="B4" t="str">
         <v>Treasurer</v>
@@ -609,15 +545,15 @@
         <v>A-701</v>
       </c>
       <c r="D4" t="str">
-        <v>+91 98200 11225</v>
+        <v/>
       </c>
       <c r="E4" t="str">
-        <v>farhan.q@example.com</v>
+        <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Meera Nair</v>
+        <v/>
       </c>
       <c r="B5" t="str">
         <v>Committee Member</v>
@@ -626,15 +562,15 @@
         <v>C-203</v>
       </c>
       <c r="D5" t="str">
-        <v>+91 98200 11226</v>
+        <v/>
       </c>
       <c r="E5" t="str">
-        <v>meera.nair@example.com</v>
+        <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Harpreet Singh</v>
+        <v/>
       </c>
       <c r="B6" t="str">
         <v>Committee Member</v>
@@ -643,7 +579,7 @@
         <v>B-604</v>
       </c>
       <c r="D6" t="str">
-        <v>+91 98200 11227</v>
+        <v/>
       </c>
       <c r="E6" t="str">
         <v/>
@@ -659,6 +595,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D6"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -699,7 +641,7 @@
         <v>100</v>
       </c>
       <c r="D3" t="str">
-        <v>Kharghar station</v>
+        <v>Ich station</v>
       </c>
     </row>
     <row r="4">
@@ -721,7 +663,7 @@
         <v>Security Gate</v>
       </c>
       <c r="B5" t="str">
-        <v>Ravi Yadav</v>
+        <v/>
       </c>
       <c r="C5" t="str">
         <v>+91 90040 55501</v>
@@ -754,6 +696,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F19"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="12.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1144,7 +1094,15 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:F25"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="12.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1165,15 +1123,6 @@
       <c r="F1" t="str">
         <v>Type</v>
       </c>
-      <c r="G1" t="str">
-        <v>Owner Name</v>
-      </c>
-      <c r="H1" t="str">
-        <v>Owner Phone</v>
-      </c>
-      <c r="I1" t="str">
-        <v>Owner Address</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -1186,21 +1135,12 @@
         <v>A-101</v>
       </c>
       <c r="D2" t="str">
-        <v>+91 98330 40011</v>
+        <v/>
       </c>
       <c r="E2" t="str">
-        <v>anil.k@example.com</v>
+        <v/>
       </c>
       <c r="F2" t="str">
-        <v>Owner</v>
-      </c>
-      <c r="G2" t="str">
-        <v/>
-      </c>
-      <c r="H2" t="str">
-        <v/>
-      </c>
-      <c r="I2" t="str">
         <v/>
       </c>
     </row>
@@ -1215,21 +1155,12 @@
         <v>A-202</v>
       </c>
       <c r="D3" t="str">
-        <v>+91 98330 40012</v>
+        <v/>
       </c>
       <c r="E3" t="str">
-        <v>priya.r@example.com</v>
+        <v/>
       </c>
       <c r="F3" t="str">
-        <v>Owner</v>
-      </c>
-      <c r="G3" t="str">
-        <v/>
-      </c>
-      <c r="H3" t="str">
-        <v/>
-      </c>
-      <c r="I3" t="str">
         <v/>
       </c>
     </row>
@@ -1244,22 +1175,13 @@
         <v>A-305</v>
       </c>
       <c r="D4" t="str">
-        <v>+91 98330 40013</v>
+        <v/>
       </c>
       <c r="E4" t="str">
         <v/>
       </c>
       <c r="F4" t="str">
-        <v>Tenant</v>
-      </c>
-      <c r="G4" t="str">
-        <v>Sanjay Kulkarni</v>
-      </c>
-      <c r="H4" t="str">
-        <v>+91 98200 44001</v>
-      </c>
-      <c r="I4" t="str">
-        <v>Flat 9, Sunrise Apartments, Aundh, Pune 411007</v>
+        <v/>
       </c>
     </row>
     <row r="5">
@@ -1273,21 +1195,12 @@
         <v>A-506</v>
       </c>
       <c r="D5" t="str">
-        <v>+91 98330 40014</v>
+        <v/>
       </c>
       <c r="E5" t="str">
-        <v>kavita.j@example.com</v>
+        <v/>
       </c>
       <c r="F5" t="str">
-        <v>Owner</v>
-      </c>
-      <c r="G5" t="str">
-        <v/>
-      </c>
-      <c r="H5" t="str">
-        <v/>
-      </c>
-      <c r="I5" t="str">
         <v/>
       </c>
     </row>
@@ -1302,21 +1215,12 @@
         <v>A-608</v>
       </c>
       <c r="D6" t="str">
-        <v>+91 98330 40023</v>
+        <v/>
       </c>
       <c r="E6" t="str">
         <v/>
       </c>
       <c r="F6" t="str">
-        <v>Owner</v>
-      </c>
-      <c r="G6" t="str">
-        <v/>
-      </c>
-      <c r="H6" t="str">
-        <v/>
-      </c>
-      <c r="I6" t="str">
         <v/>
       </c>
     </row>
@@ -1331,21 +1235,12 @@
         <v>B-201</v>
       </c>
       <c r="D7" t="str">
-        <v>+91 98330 40015</v>
+        <v/>
       </c>
       <c r="E7" t="str">
         <v/>
       </c>
       <c r="F7" t="str">
-        <v>Owner</v>
-      </c>
-      <c r="G7" t="str">
-        <v/>
-      </c>
-      <c r="H7" t="str">
-        <v/>
-      </c>
-      <c r="I7" t="str">
         <v/>
       </c>
     </row>
@@ -1360,21 +1255,12 @@
         <v>B-302</v>
       </c>
       <c r="D8" t="str">
-        <v>+91 98330 40016</v>
+        <v/>
       </c>
       <c r="E8" t="str">
-        <v>deepa.c@example.com</v>
+        <v/>
       </c>
       <c r="F8" t="str">
-        <v>Owner</v>
-      </c>
-      <c r="G8" t="str">
-        <v/>
-      </c>
-      <c r="H8" t="str">
-        <v/>
-      </c>
-      <c r="I8" t="str">
         <v/>
       </c>
     </row>
@@ -1389,22 +1275,13 @@
         <v>B-403</v>
       </c>
       <c r="D9" t="str">
-        <v>+91 98330 40017</v>
+        <v/>
       </c>
       <c r="E9" t="str">
         <v/>
       </c>
       <c r="F9" t="str">
-        <v>Tenant</v>
-      </c>
-      <c r="G9" t="str">
-        <v>Rajesh Menon</v>
-      </c>
-      <c r="H9" t="str">
-        <v>+91 98200 44002</v>
-      </c>
-      <c r="I9" t="str">
-        <v>B-201, Green Valley Residency (resident owner)</v>
+        <v/>
       </c>
     </row>
     <row r="10">
@@ -1418,21 +1295,12 @@
         <v>B-505</v>
       </c>
       <c r="D10" t="str">
-        <v>+91 98330 40018</v>
+        <v/>
       </c>
       <c r="E10" t="str">
-        <v>nisha.p@example.com</v>
+        <v/>
       </c>
       <c r="F10" t="str">
-        <v>Owner</v>
-      </c>
-      <c r="G10" t="str">
-        <v/>
-      </c>
-      <c r="H10" t="str">
-        <v/>
-      </c>
-      <c r="I10" t="str">
         <v/>
       </c>
     </row>
@@ -1447,21 +1315,12 @@
         <v>B-707</v>
       </c>
       <c r="D11" t="str">
-        <v>+91 98330 40024</v>
+        <v/>
       </c>
       <c r="E11" t="str">
         <v/>
       </c>
       <c r="F11" t="str">
-        <v>Owner</v>
-      </c>
-      <c r="G11" t="str">
-        <v/>
-      </c>
-      <c r="H11" t="str">
-        <v/>
-      </c>
-      <c r="I11" t="str">
         <v/>
       </c>
     </row>
@@ -1476,21 +1335,12 @@
         <v>C-102</v>
       </c>
       <c r="D12" t="str">
-        <v>+91 98330 40019</v>
+        <v/>
       </c>
       <c r="E12" t="str">
         <v/>
       </c>
       <c r="F12" t="str">
-        <v>Owner</v>
-      </c>
-      <c r="G12" t="str">
-        <v/>
-      </c>
-      <c r="H12" t="str">
-        <v/>
-      </c>
-      <c r="I12" t="str">
         <v/>
       </c>
     </row>
@@ -1505,22 +1355,13 @@
         <v>C-304</v>
       </c>
       <c r="D13" t="str">
-        <v>+91 98330 40020</v>
+        <v/>
       </c>
       <c r="E13" t="str">
-        <v>ayesha.k@example.com</v>
+        <v/>
       </c>
       <c r="F13" t="str">
-        <v>Tenant</v>
-      </c>
-      <c r="G13" t="str">
-        <v>Farida Merchant</v>
-      </c>
-      <c r="H13" t="str">
-        <v>+91 98200 44003</v>
-      </c>
-      <c r="I13" t="str">
-        <v>22 Peddar Road, Mumbai 400026</v>
+        <v/>
       </c>
     </row>
     <row r="14">
@@ -1534,21 +1375,12 @@
         <v>C-405</v>
       </c>
       <c r="D14" t="str">
-        <v>+91 98330 40021</v>
+        <v/>
       </c>
       <c r="E14" t="str">
         <v/>
       </c>
       <c r="F14" t="str">
-        <v>Owner</v>
-      </c>
-      <c r="G14" t="str">
-        <v/>
-      </c>
-      <c r="H14" t="str">
-        <v/>
-      </c>
-      <c r="I14" t="str">
         <v/>
       </c>
     </row>
@@ -1563,21 +1395,12 @@
         <v>C-506</v>
       </c>
       <c r="D15" t="str">
-        <v>+91 98330 40022</v>
+        <v/>
       </c>
       <c r="E15" t="str">
-        <v>lakshmi.s@example.com</v>
+        <v/>
       </c>
       <c r="F15" t="str">
-        <v>Owner</v>
-      </c>
-      <c r="G15" t="str">
-        <v/>
-      </c>
-      <c r="H15" t="str">
-        <v/>
-      </c>
-      <c r="I15" t="str">
         <v/>
       </c>
     </row>
@@ -1592,27 +1415,198 @@
         <v>C-608</v>
       </c>
       <c r="D16" t="str">
-        <v>+91 98330 40025</v>
+        <v/>
       </c>
       <c r="E16" t="str">
-        <v>tanvi.m@example.com</v>
+        <v/>
       </c>
       <c r="F16" t="str">
-        <v>Owner</v>
-      </c>
-      <c r="G16" t="str">
-        <v/>
-      </c>
-      <c r="H16" t="str">
-        <v/>
-      </c>
-      <c r="I16" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Narendrakumar heda</v>
+      </c>
+      <c r="B17" t="str">
+        <v>B</v>
+      </c>
+      <c r="C17" t="str">
+        <v>11</v>
+      </c>
+      <c r="D17" t="str">
+        <v>8793109590</v>
+      </c>
+      <c r="E17" t="str">
+        <v/>
+      </c>
+      <c r="F17" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Bhavesh Rajeshkumar Sarda</v>
+      </c>
+      <c r="B18" t="str">
+        <v>B</v>
+      </c>
+      <c r="C18" t="str">
+        <v>B-2</v>
+      </c>
+      <c r="D18" t="str">
+        <v>8482996010</v>
+      </c>
+      <c r="E18" t="str">
+        <v>bhaveshsarda2004@gmail.com</v>
+      </c>
+      <c r="F18" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Sagar Agarwal</v>
+      </c>
+      <c r="B19" t="str">
+        <v>A</v>
+      </c>
+      <c r="C19" t="str">
+        <v>A - 2</v>
+      </c>
+      <c r="D19" t="str">
+        <v>7350665037</v>
+      </c>
+      <c r="E19" t="str">
+        <v>agarwalsagar016@gmail.com</v>
+      </c>
+      <c r="F19" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>Rahul Pareek</v>
+      </c>
+      <c r="B20" t="str">
+        <v>B</v>
+      </c>
+      <c r="C20" t="str">
+        <v>9</v>
+      </c>
+      <c r="D20" t="str">
+        <v>9156704040</v>
+      </c>
+      <c r="E20" t="str">
+        <v>rahulpareek3366@gmail.com</v>
+      </c>
+      <c r="F20" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Shrihari Narayan Makote</v>
+      </c>
+      <c r="B21" t="str">
+        <v>D</v>
+      </c>
+      <c r="C21" t="str">
+        <v>12</v>
+      </c>
+      <c r="D21" t="str">
+        <v>9922497427</v>
+      </c>
+      <c r="E21" t="str">
+        <v>shriharimakote70@gmail.com</v>
+      </c>
+      <c r="F21" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>Ramdev Rathi</v>
+      </c>
+      <c r="B22" t="str">
+        <v>C</v>
+      </c>
+      <c r="C22" t="str">
+        <v>C2-C3</v>
+      </c>
+      <c r="D22" t="str">
+        <v>9422423985</v>
+      </c>
+      <c r="E22" t="str">
+        <v/>
+      </c>
+      <c r="F22" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>Pradeep Jhunjhunwala</v>
+      </c>
+      <c r="B23" t="str">
+        <v>A</v>
+      </c>
+      <c r="C23" t="str">
+        <v>A-10</v>
+      </c>
+      <c r="D23" t="str">
+        <v>9922114900</v>
+      </c>
+      <c r="E23" t="str">
+        <v>cool16yash@gmail.com</v>
+      </c>
+      <c r="F23" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>Harishkumar Bharatkumar</v>
+      </c>
+      <c r="B24" t="str">
+        <v>C</v>
+      </c>
+      <c r="C24" t="str">
+        <v>C-14</v>
+      </c>
+      <c r="D24" t="str">
+        <v>7019426263</v>
+      </c>
+      <c r="E24" t="str">
+        <v/>
+      </c>
+      <c r="F24" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>Laxmi kant balkrishan malpani</v>
+      </c>
+      <c r="B25" t="str">
+        <v>A</v>
+      </c>
+      <c r="C25" t="str">
+        <v>A/1</v>
+      </c>
+      <c r="D25" t="str">
+        <v>9372281026</v>
+      </c>
+      <c r="E25" t="str">
+        <v/>
+      </c>
+      <c r="F25" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F25"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1620,6 +1614,13 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E5"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1711,4 +1712,175 @@
     <ignoredError numberStoredAsText="1" sqref="A1:E5"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D11"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Service</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Contact</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Phone</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Notes</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Plumber</v>
+      </c>
+      <c r="B2" t="str">
+        <v/>
+      </c>
+      <c r="C2" t="str">
+        <v/>
+      </c>
+      <c r="D2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Electrician</v>
+      </c>
+      <c r="B3" t="str">
+        <v/>
+      </c>
+      <c r="C3" t="str">
+        <v/>
+      </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Lift Technician</v>
+      </c>
+      <c r="B4" t="str">
+        <v/>
+      </c>
+      <c r="C4" t="str">
+        <v/>
+      </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Pest Control</v>
+      </c>
+      <c r="B5" t="str">
+        <v/>
+      </c>
+      <c r="C5" t="str">
+        <v/>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Housekeeping</v>
+      </c>
+      <c r="B6" t="str">
+        <v/>
+      </c>
+      <c r="C6" t="str">
+        <v/>
+      </c>
+      <c r="D6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Water Tanker</v>
+      </c>
+      <c r="B7" t="str">
+        <v/>
+      </c>
+      <c r="C7" t="str">
+        <v/>
+      </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Electricity Board</v>
+      </c>
+      <c r="B8" t="str">
+        <v/>
+      </c>
+      <c r="C8" t="str">
+        <v/>
+      </c>
+      <c r="D8" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Gas Agency</v>
+      </c>
+      <c r="B9" t="str">
+        <v/>
+      </c>
+      <c r="C9" t="str">
+        <v/>
+      </c>
+      <c r="D9" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Society Manager</v>
+      </c>
+      <c r="B10" t="str">
+        <v/>
+      </c>
+      <c r="C10" t="str">
+        <v/>
+      </c>
+      <c r="D10" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Accountant</v>
+      </c>
+      <c r="B11" t="str">
+        <v/>
+      </c>
+      <c r="C11" t="str">
+        <v/>
+      </c>
+      <c r="D11" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:D11"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Update directory data (73 rows)
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -403,7 +403,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B8"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -465,9 +465,17 @@
         <v>NBOM/HSG/1284/2009</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Theme</v>
+      </c>
+      <c r="B8" t="str">
+        <v>slate</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B8"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update directory data (90 rows)
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -10,6 +10,8 @@
     <sheet name="Residents" sheetId="5" r:id="rId5"/>
     <sheet name="Documents" sheetId="6" r:id="rId6"/>
     <sheet name="Services" sheetId="7" r:id="rId7"/>
+    <sheet name="_Private" sheetId="8" r:id="rId8"/>
+    <sheet name="_Read me" sheetId="9" r:id="rId9"/>
   </sheets>
 </workbook>
 </file>
@@ -403,10 +405,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:C17"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="34.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -416,13 +419,19 @@
       <c r="B1" t="str">
         <v>Value</v>
       </c>
+      <c r="C1" t="str">
+        <v>What it does / यह क्या करता है</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
         <v>Society Name</v>
       </c>
       <c r="B2" t="str">
-        <v>Laxmi venkatesh Nagar</v>
+        <v>LAXMI VENKATESH NAGAR</v>
+      </c>
+      <c r="C2" t="str">
+        <v>सोसाइटी का नाम — बड़े शीर्षक में दिखेगा</v>
       </c>
     </row>
     <row r="3">
@@ -430,7 +439,10 @@
         <v>Tagline</v>
       </c>
       <c r="B3" t="str">
-        <v>Best Housing Society in Ichalkaranji</v>
+        <v>The Best Society in ICHALKARANJI</v>
+      </c>
+      <c r="C3" t="str">
+        <v>उपशीर्षक</v>
       </c>
     </row>
     <row r="4">
@@ -440,13 +452,19 @@
       <c r="B4" t="str">
         <v>Old chandur road</v>
       </c>
+      <c r="C4" t="str">
+        <v>पता</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
         <v>City</v>
       </c>
       <c r="B5" t="str">
-        <v>ichalkaranji</v>
+        <v>Ichalkaranji</v>
+      </c>
+      <c r="C5" t="str">
+        <v>शहर</v>
       </c>
     </row>
     <row r="6">
@@ -456,33 +474,141 @@
       <c r="B6" t="str">
         <v>416115</v>
       </c>
+      <c r="C6" t="str">
+        <v>पिन कोड</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
         <v>Registration No</v>
       </c>
       <c r="B7" t="str">
-        <v>NBOM/HSG/1284/2009</v>
+        <v/>
+      </c>
+      <c r="C7" t="str">
+        <v>पंजीकरण संख्या — नीचे फुटर में</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
+        <v>Logo</v>
+      </c>
+      <c r="B8" t="str">
+        <v/>
+      </c>
+      <c r="C8" t="str">
+        <v>वैकल्पिक: लोगो की इमेज URL</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Confidential Notice</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Please do not forward this link or share these details with anyone outside the society.</v>
+      </c>
+      <c r="C9" t="str">
+        <v>ऊपर दिखने वाली चेतावनी (अंग्रेज़ी)</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Confidential HI</v>
+      </c>
+      <c r="B10" t="str">
+        <v>कृपया यह लिंक या विवरण सोसाइटी के बाहर किसी के साथ साझा न करें।</v>
+      </c>
+      <c r="C10" t="str">
+        <v>वही चेतावनी हिंदी में</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
         <v>Theme</v>
       </c>
-      <c r="B8" t="str">
-        <v>paper</v>
+      <c r="B11" t="str">
+        <v>Paper</v>
+      </c>
+      <c r="C11" t="str">
+        <v>navy, forest, plum, slate, sunset, ocean, paper</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Hindi: Committee</v>
+      </c>
+      <c r="B12" t="str">
+        <v>समिति</v>
+      </c>
+      <c r="C12" t="str">
+        <v>हिंदी में अनुभाग का नाम</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Hindi: Emergency</v>
+      </c>
+      <c r="B13" t="str">
+        <v>आपातकालीन संपर्क</v>
+      </c>
+      <c r="C13" t="str">
+        <v>हिंदी में अनुभाग का नाम</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Hindi: Services &amp; Help</v>
+      </c>
+      <c r="B14" t="str">
+        <v>सेवाएँ और सहायता</v>
+      </c>
+      <c r="C14" t="str">
+        <v>हिंदी में अनुभाग का नाम</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Hindi: Residents</v>
+      </c>
+      <c r="B15" t="str">
+        <v>निवासी</v>
+      </c>
+      <c r="C15" t="str">
+        <v>हिंदी में अनुभाग का नाम</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>Hindi: Documents</v>
+      </c>
+      <c r="B16" t="str">
+        <v>दस्तावेज़</v>
+      </c>
+      <c r="C16" t="str">
+        <v>हिंदी में अनुभाग का नाम</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Note: Services &amp; Help</v>
+      </c>
+      <c r="B17" t="str">
+        <v>These contacts are collected from members. They have not been verified or endorsed. Please check credentials and agree charges before engaging anyone — you do so at your own risk.</v>
+      </c>
+      <c r="C17" t="str">
+        <v>उस अनुभाग के नीचे दिखने वाली चेतावनी</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C17"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E3"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -516,7 +642,7 @@
         <v>Chairman</v>
       </c>
       <c r="C2" t="str">
-        <v>A-402</v>
+        <v/>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -533,76 +659,25 @@
         <v>Hon. Secretary</v>
       </c>
       <c r="C3" t="str">
-        <v>B-105</v>
+        <v/>
       </c>
       <c r="D3" t="str">
         <v/>
       </c>
       <c r="E3" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v/>
-      </c>
-      <c r="B4" t="str">
-        <v>Treasurer</v>
-      </c>
-      <c r="C4" t="str">
-        <v>A-701</v>
-      </c>
-      <c r="D4" t="str">
-        <v/>
-      </c>
-      <c r="E4" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v/>
-      </c>
-      <c r="B5" t="str">
-        <v>Committee Member</v>
-      </c>
-      <c r="C5" t="str">
-        <v>C-203</v>
-      </c>
-      <c r="D5" t="str">
-        <v/>
-      </c>
-      <c r="E5" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v/>
-      </c>
-      <c r="B6" t="str">
-        <v>Committee Member</v>
-      </c>
-      <c r="C6" t="str">
-        <v>B-604</v>
-      </c>
-      <c r="D6" t="str">
-        <v/>
-      </c>
-      <c r="E6" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D5"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -649,7 +724,7 @@
         <v>100</v>
       </c>
       <c r="D3" t="str">
-        <v>Ich station</v>
+        <v/>
       </c>
     </row>
     <row r="4">
@@ -663,7 +738,7 @@
         <v>101</v>
       </c>
       <c r="D4" t="str">
-        <v>Toll free, 24x7</v>
+        <v/>
       </c>
     </row>
     <row r="5">
@@ -671,32 +746,18 @@
         <v>Security Gate</v>
       </c>
       <c r="B5" t="str">
-        <v/>
+        <v>Example Name</v>
       </c>
       <c r="C5" t="str">
-        <v>+91 90040 55501</v>
+        <v>9.1E+12</v>
       </c>
       <c r="D5" t="str">
         <v>Main gate, 24x7</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>Ndrf Helpline</v>
-      </c>
-      <c r="B6" t="str">
-        <v/>
-      </c>
-      <c r="C6" t="str">
-        <v>108</v>
-      </c>
-      <c r="D6" t="str">
-        <v>Disaster response</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D5"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -747,7 +808,7 @@
         <v>8 AM – 8 PM, on call</v>
       </c>
       <c r="E2" t="str">
-        <v>+91 90040 55511</v>
+        <v/>
       </c>
       <c r="F2" t="str">
         <v>Parts charged separately</v>
@@ -767,7 +828,7 @@
         <v>9 AM – 8 PM, on call</v>
       </c>
       <c r="E3" t="str">
-        <v>+91 90040 55512</v>
+        <v/>
       </c>
       <c r="F3" t="str">
         <v>Wiring, fans, MCB</v>
@@ -775,7 +836,7 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Salim Ansari</v>
+        <v>Jangid</v>
       </c>
       <c r="B4" t="str">
         <v>Carpenter</v>
@@ -787,7 +848,7 @@
         <v>On call</v>
       </c>
       <c r="E4" t="str">
-        <v>+91 90210 33009</v>
+        <v/>
       </c>
       <c r="F4" t="str">
         <v>Furniture repair and fittings</v>
@@ -807,7 +868,7 @@
         <v>4-hour response</v>
       </c>
       <c r="E5" t="str">
-        <v>+91 90040 55513</v>
+        <v/>
       </c>
       <c r="F5" t="str">
         <v>Report faults to the manager first</v>
@@ -827,7 +888,7 @@
         <v>By appointment</v>
       </c>
       <c r="E6" t="str">
-        <v>+91 90040 55514</v>
+        <v/>
       </c>
       <c r="F6" t="str">
         <v>Quarterly society drive is free</v>
@@ -847,7 +908,7 @@
         <v>6 AM – 2 PM</v>
       </c>
       <c r="E7" t="str">
-        <v>+91 90040 55515</v>
+        <v/>
       </c>
       <c r="F7" t="str">
         <v>Common areas and staircases</v>
@@ -867,7 +928,7 @@
         <v>Tue &amp; Sat mornings</v>
       </c>
       <c r="E8" t="str">
-        <v>+91 90210 33010</v>
+        <v/>
       </c>
       <c r="F8" t="str">
         <v>Balcony and terrace plants</v>
@@ -887,7 +948,7 @@
         <v>Same-day delivery</v>
       </c>
       <c r="E9" t="str">
-        <v>+91 90040 55521</v>
+        <v/>
       </c>
       <c r="F9" t="str">
         <v>10,000 litre tanker</v>
@@ -907,7 +968,7 @@
         <v>24x7 helpline</v>
       </c>
       <c r="E10" t="str">
-        <v>1912</v>
+        <v/>
       </c>
       <c r="F10" t="str">
         <v>Outages and meter faults</v>
@@ -927,7 +988,7 @@
         <v>24x7 for leaks</v>
       </c>
       <c r="E11" t="str">
-        <v>+91 90040 55522</v>
+        <v/>
       </c>
       <c r="F11" t="str">
         <v>Leak helpline 1800 22 9944</v>
@@ -947,7 +1008,7 @@
         <v>Mon–Sat, 10 AM – 6 PM</v>
       </c>
       <c r="E12" t="str">
-        <v>+91 90040 55531</v>
+        <v/>
       </c>
       <c r="F12" t="str">
         <v>Maintenance bills, NOCs, complaints</v>
@@ -967,7 +1028,7 @@
         <v>Tue &amp; Thu, 4 PM – 7 PM</v>
       </c>
       <c r="E13" t="str">
-        <v>+91 90040 55532</v>
+        <v/>
       </c>
       <c r="F13" t="str">
         <v>Dues, receipts, statements</v>
@@ -987,7 +1048,7 @@
         <v>7 AM – 11 AM</v>
       </c>
       <c r="E14" t="str">
-        <v>+91 90210 33001</v>
+        <v/>
       </c>
       <c r="F14" t="str">
         <v>Sweeping, mopping, utensils</v>
@@ -1007,7 +1068,7 @@
         <v>6 AM – 10 AM</v>
       </c>
       <c r="E15" t="str">
-        <v>+91 90210 33002</v>
+        <v/>
       </c>
       <c r="F15" t="str">
         <v>Also irons clothes on request</v>
@@ -1027,7 +1088,7 @@
         <v>11 AM – 2 PM</v>
       </c>
       <c r="E16" t="str">
-        <v>+91 90210 33005</v>
+        <v/>
       </c>
       <c r="F16" t="str">
         <v>Vegetarian, two meals a day</v>
@@ -1035,7 +1096,7 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Imran Shaikh</v>
+        <v>ganesh raju</v>
       </c>
       <c r="B17" t="str">
         <v>Car Cleaning</v>
@@ -1047,7 +1108,7 @@
         <v>6 AM – 9 AM</v>
       </c>
       <c r="E17" t="str">
-        <v>+91 90210 33006</v>
+        <v/>
       </c>
       <c r="F17" t="str">
         <v>Daily wash, interior weekly</v>
@@ -1067,7 +1128,7 @@
         <v>By appointment</v>
       </c>
       <c r="E18" t="str">
-        <v>+91 90210 33007</v>
+        <v/>
       </c>
       <c r="F18" t="str">
         <v>Local trips, holds a valid licence</v>
@@ -1087,7 +1148,7 @@
         <v>Flexible</v>
       </c>
       <c r="E19" t="str">
-        <v>+91 90210 33008</v>
+        <v/>
       </c>
       <c r="F19" t="str">
         <v>Experienced with toddlers</v>
@@ -1102,7 +1163,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:R21"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1110,6 +1171,18 @@
     <col min="4" max="4" width="12.83203125" customWidth="1"/>
     <col min="5" max="5" width="12.83203125" customWidth="1"/>
     <col min="6" max="6" width="12.83203125" customWidth="1"/>
+    <col min="7" max="7" width="15.83203125" customWidth="1"/>
+    <col min="8" max="8" width="21.83203125" customWidth="1"/>
+    <col min="9" max="9" width="14.83203125" customWidth="1"/>
+    <col min="10" max="10" width="16.83203125" customWidth="1"/>
+    <col min="11" max="11" width="16.83203125" customWidth="1"/>
+    <col min="12" max="12" width="14.83203125" customWidth="1"/>
+    <col min="13" max="13" width="12.83203125" customWidth="1"/>
+    <col min="14" max="14" width="13.83203125" customWidth="1"/>
+    <col min="15" max="15" width="12.83203125" customWidth="1"/>
+    <col min="16" max="16" width="14.83203125" customWidth="1"/>
+    <col min="17" max="17" width="15.83203125" customWidth="1"/>
+    <col min="18" max="18" width="17.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1131,497 +1204,1173 @@
       <c r="F1" t="str">
         <v>Type</v>
       </c>
+      <c r="G1" t="str">
+        <v>Blood Group</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Emergency Contact</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Vehicle No</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Vehicle Type</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Parking Slot</v>
+      </c>
+      <c r="L1" t="str">
+        <v>Profession</v>
+      </c>
+      <c r="M1" t="str">
+        <v>Language</v>
+      </c>
+      <c r="N1" t="str">
+        <v>Occupants</v>
+      </c>
+      <c r="O1" t="str">
+        <v>Pets</v>
+      </c>
+      <c r="P1" t="str">
+        <v>Owner Name</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>Owner Phone</v>
+      </c>
+      <c r="R1" t="str">
+        <v>Owner Address</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Anil Kulkarni</v>
+        <v>Test Name</v>
       </c>
       <c r="B2" t="str">
-        <v>A</v>
+        <v>B</v>
       </c>
       <c r="C2" t="str">
-        <v>A-101</v>
+        <v>10</v>
       </c>
       <c r="D2" t="str">
-        <v/>
+        <v>9876543210</v>
       </c>
       <c r="E2" t="str">
-        <v/>
+        <v>abc@xyz.com</v>
       </c>
       <c r="F2" t="str">
+        <v>owner</v>
+      </c>
+      <c r="G2" t="str">
+        <v>O+</v>
+      </c>
+      <c r="H2" t="str">
+        <v>Relative name, +91 98220 11111</v>
+      </c>
+      <c r="I2" t="str">
+        <v>MH-09-AB-1234</v>
+      </c>
+      <c r="J2" t="str">
+        <v>Car</v>
+      </c>
+      <c r="K2" t="str">
+        <v>P-12</v>
+      </c>
+      <c r="L2" t="str">
+        <v>Doctor</v>
+      </c>
+      <c r="M2" t="str">
+        <v>Marathi</v>
+      </c>
+      <c r="N2" t="str">
+        <v>4</v>
+      </c>
+      <c r="O2" t="str">
+        <v/>
+      </c>
+      <c r="P2" t="str">
+        <v/>
+      </c>
+      <c r="Q2" t="str">
+        <v/>
+      </c>
+      <c r="R2" t="str">
         <v/>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Priya Raghavan</v>
+        <v>Test Name - Tenant</v>
       </c>
       <c r="B3" t="str">
         <v>A</v>
       </c>
       <c r="C3" t="str">
-        <v>A-202</v>
+        <v>2</v>
       </c>
       <c r="D3" t="str">
-        <v/>
+        <v>9876543210</v>
       </c>
       <c r="E3" t="str">
-        <v/>
+        <v>abc@xyz.com</v>
       </c>
       <c r="F3" t="str">
-        <v/>
+        <v>tenant</v>
+      </c>
+      <c r="G3" t="str">
+        <v>A+</v>
+      </c>
+      <c r="H3" t="str">
+        <v/>
+      </c>
+      <c r="I3" t="str">
+        <v>MH-09-CD-5678</v>
+      </c>
+      <c r="J3" t="str">
+        <v>Two-wheeler</v>
+      </c>
+      <c r="K3" t="str">
+        <v>P-31</v>
+      </c>
+      <c r="L3" t="str">
+        <v>Teacher</v>
+      </c>
+      <c r="M3" t="str">
+        <v>Hindi</v>
+      </c>
+      <c r="N3" t="str">
+        <v>2</v>
+      </c>
+      <c r="O3" t="str">
+        <v>1 cat</v>
+      </c>
+      <c r="P3" t="str">
+        <v>Flat Owner Name</v>
+      </c>
+      <c r="Q3" t="str">
+        <v>+91 98200 44002</v>
+      </c>
+      <c r="R3" t="str">
+        <v>Owner's address, city</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Imran Shaikh</v>
+        <v>Narendrakumar heda</v>
       </c>
       <c r="B4" t="str">
-        <v>A</v>
+        <v>B</v>
       </c>
       <c r="C4" t="str">
-        <v>A-305</v>
+        <v>11</v>
       </c>
       <c r="D4" t="str">
-        <v/>
+        <v>8793109590</v>
       </c>
       <c r="E4" t="str">
         <v/>
       </c>
       <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4" t="str">
+        <v/>
+      </c>
+      <c r="H4" t="str">
+        <v/>
+      </c>
+      <c r="I4" t="str">
+        <v/>
+      </c>
+      <c r="J4" t="str">
+        <v/>
+      </c>
+      <c r="K4" t="str">
+        <v/>
+      </c>
+      <c r="L4" t="str">
+        <v/>
+      </c>
+      <c r="M4" t="str">
+        <v/>
+      </c>
+      <c r="N4" t="str">
+        <v/>
+      </c>
+      <c r="O4" t="str">
+        <v/>
+      </c>
+      <c r="P4" t="str">
+        <v/>
+      </c>
+      <c r="Q4" t="str">
+        <v/>
+      </c>
+      <c r="R4" t="str">
         <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Kavita Joshi</v>
+        <v>Bhavesh Rajeshkumar Sarda</v>
       </c>
       <c r="B5" t="str">
-        <v>A</v>
+        <v>B</v>
       </c>
       <c r="C5" t="str">
-        <v>A-506</v>
+        <v>B-2</v>
       </c>
       <c r="D5" t="str">
-        <v/>
+        <v>8482996010</v>
       </c>
       <c r="E5" t="str">
-        <v/>
+        <v>bhaveshsarda2004@gmail.com</v>
       </c>
       <c r="F5" t="str">
+        <v/>
+      </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
+      <c r="H5" t="str">
+        <v/>
+      </c>
+      <c r="I5" t="str">
+        <v/>
+      </c>
+      <c r="J5" t="str">
+        <v/>
+      </c>
+      <c r="K5" t="str">
+        <v/>
+      </c>
+      <c r="L5" t="str">
+        <v/>
+      </c>
+      <c r="M5" t="str">
+        <v/>
+      </c>
+      <c r="N5" t="str">
+        <v/>
+      </c>
+      <c r="O5" t="str">
+        <v/>
+      </c>
+      <c r="P5" t="str">
+        <v/>
+      </c>
+      <c r="Q5" t="str">
+        <v/>
+      </c>
+      <c r="R5" t="str">
         <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Rohan Bhatia</v>
+        <v>Sagar Agarwal</v>
       </c>
       <c r="B6" t="str">
         <v>A</v>
       </c>
       <c r="C6" t="str">
-        <v>A-608</v>
+        <v>A - 2</v>
       </c>
       <c r="D6" t="str">
-        <v/>
+        <v>7350665037</v>
       </c>
       <c r="E6" t="str">
-        <v/>
+        <v>agarwalsagar016@gmail.com</v>
       </c>
       <c r="F6" t="str">
+        <v/>
+      </c>
+      <c r="G6" t="str">
+        <v/>
+      </c>
+      <c r="H6" t="str">
+        <v/>
+      </c>
+      <c r="I6" t="str">
+        <v/>
+      </c>
+      <c r="J6" t="str">
+        <v/>
+      </c>
+      <c r="K6" t="str">
+        <v/>
+      </c>
+      <c r="L6" t="str">
+        <v/>
+      </c>
+      <c r="M6" t="str">
+        <v/>
+      </c>
+      <c r="N6" t="str">
+        <v/>
+      </c>
+      <c r="O6" t="str">
+        <v/>
+      </c>
+      <c r="P6" t="str">
+        <v/>
+      </c>
+      <c r="Q6" t="str">
+        <v/>
+      </c>
+      <c r="R6" t="str">
         <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Rajesh Menon</v>
+        <v>Rahul Pareek</v>
       </c>
       <c r="B7" t="str">
         <v>B</v>
       </c>
       <c r="C7" t="str">
-        <v>B-201</v>
+        <v>9</v>
       </c>
       <c r="D7" t="str">
-        <v/>
+        <v>9156704040</v>
       </c>
       <c r="E7" t="str">
-        <v/>
+        <v>rahulpareek3366@gmail.com</v>
       </c>
       <c r="F7" t="str">
+        <v/>
+      </c>
+      <c r="G7" t="str">
+        <v/>
+      </c>
+      <c r="H7" t="str">
+        <v/>
+      </c>
+      <c r="I7" t="str">
+        <v/>
+      </c>
+      <c r="J7" t="str">
+        <v/>
+      </c>
+      <c r="K7" t="str">
+        <v/>
+      </c>
+      <c r="L7" t="str">
+        <v/>
+      </c>
+      <c r="M7" t="str">
+        <v/>
+      </c>
+      <c r="N7" t="str">
+        <v/>
+      </c>
+      <c r="O7" t="str">
+        <v/>
+      </c>
+      <c r="P7" t="str">
+        <v/>
+      </c>
+      <c r="Q7" t="str">
+        <v/>
+      </c>
+      <c r="R7" t="str">
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Deepa Chatterjee</v>
+        <v>Shrihari Narayan Makote</v>
       </c>
       <c r="B8" t="str">
-        <v>B</v>
+        <v>D</v>
       </c>
       <c r="C8" t="str">
-        <v>B-302</v>
+        <v>12</v>
       </c>
       <c r="D8" t="str">
-        <v/>
+        <v>9922497427</v>
       </c>
       <c r="E8" t="str">
-        <v/>
+        <v>shriharimakote70@gmail.com</v>
       </c>
       <c r="F8" t="str">
+        <v/>
+      </c>
+      <c r="G8" t="str">
+        <v/>
+      </c>
+      <c r="H8" t="str">
+        <v/>
+      </c>
+      <c r="I8" t="str">
+        <v/>
+      </c>
+      <c r="J8" t="str">
+        <v/>
+      </c>
+      <c r="K8" t="str">
+        <v/>
+      </c>
+      <c r="L8" t="str">
+        <v/>
+      </c>
+      <c r="M8" t="str">
+        <v/>
+      </c>
+      <c r="N8" t="str">
+        <v/>
+      </c>
+      <c r="O8" t="str">
+        <v/>
+      </c>
+      <c r="P8" t="str">
+        <v/>
+      </c>
+      <c r="Q8" t="str">
+        <v/>
+      </c>
+      <c r="R8" t="str">
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Vikram Rathore</v>
+        <v>Ramdev Rathi</v>
       </c>
       <c r="B9" t="str">
-        <v>B</v>
+        <v>C</v>
       </c>
       <c r="C9" t="str">
-        <v>B-403</v>
+        <v>C2-C3</v>
       </c>
       <c r="D9" t="str">
-        <v/>
+        <v>9422423985</v>
       </c>
       <c r="E9" t="str">
         <v/>
       </c>
       <c r="F9" t="str">
+        <v/>
+      </c>
+      <c r="G9" t="str">
+        <v/>
+      </c>
+      <c r="H9" t="str">
+        <v/>
+      </c>
+      <c r="I9" t="str">
+        <v/>
+      </c>
+      <c r="J9" t="str">
+        <v/>
+      </c>
+      <c r="K9" t="str">
+        <v/>
+      </c>
+      <c r="L9" t="str">
+        <v/>
+      </c>
+      <c r="M9" t="str">
+        <v/>
+      </c>
+      <c r="N9" t="str">
+        <v/>
+      </c>
+      <c r="O9" t="str">
+        <v/>
+      </c>
+      <c r="P9" t="str">
+        <v/>
+      </c>
+      <c r="Q9" t="str">
+        <v/>
+      </c>
+      <c r="R9" t="str">
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Nisha Patel</v>
+        <v>Pradeep Jhunjhunwala</v>
       </c>
       <c r="B10" t="str">
-        <v>B</v>
+        <v>A</v>
       </c>
       <c r="C10" t="str">
-        <v>B-505</v>
+        <v>A-10</v>
       </c>
       <c r="D10" t="str">
-        <v/>
+        <v>9922114900</v>
       </c>
       <c r="E10" t="str">
-        <v/>
+        <v>cool16yash@gmail.com</v>
       </c>
       <c r="F10" t="str">
+        <v/>
+      </c>
+      <c r="G10" t="str">
+        <v/>
+      </c>
+      <c r="H10" t="str">
+        <v/>
+      </c>
+      <c r="I10" t="str">
+        <v/>
+      </c>
+      <c r="J10" t="str">
+        <v/>
+      </c>
+      <c r="K10" t="str">
+        <v/>
+      </c>
+      <c r="L10" t="str">
+        <v/>
+      </c>
+      <c r="M10" t="str">
+        <v/>
+      </c>
+      <c r="N10" t="str">
+        <v/>
+      </c>
+      <c r="O10" t="str">
+        <v/>
+      </c>
+      <c r="P10" t="str">
+        <v/>
+      </c>
+      <c r="Q10" t="str">
+        <v/>
+      </c>
+      <c r="R10" t="str">
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Arjun Sethi</v>
+        <v>Harishkumar Bharatkumar</v>
       </c>
       <c r="B11" t="str">
-        <v>B</v>
+        <v>C</v>
       </c>
       <c r="C11" t="str">
-        <v>B-707</v>
+        <v>C-14</v>
       </c>
       <c r="D11" t="str">
-        <v/>
+        <v>7019426263</v>
       </c>
       <c r="E11" t="str">
         <v/>
       </c>
       <c r="F11" t="str">
+        <v/>
+      </c>
+      <c r="G11" t="str">
+        <v/>
+      </c>
+      <c r="H11" t="str">
+        <v/>
+      </c>
+      <c r="I11" t="str">
+        <v/>
+      </c>
+      <c r="J11" t="str">
+        <v/>
+      </c>
+      <c r="K11" t="str">
+        <v/>
+      </c>
+      <c r="L11" t="str">
+        <v/>
+      </c>
+      <c r="M11" t="str">
+        <v/>
+      </c>
+      <c r="N11" t="str">
+        <v/>
+      </c>
+      <c r="O11" t="str">
+        <v/>
+      </c>
+      <c r="P11" t="str">
+        <v/>
+      </c>
+      <c r="Q11" t="str">
+        <v/>
+      </c>
+      <c r="R11" t="str">
         <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Suresh Pillai</v>
+        <v>Laxmi kant balkrishan malpani</v>
       </c>
       <c r="B12" t="str">
-        <v>C</v>
+        <v>A</v>
       </c>
       <c r="C12" t="str">
-        <v>C-102</v>
+        <v>A/1</v>
       </c>
       <c r="D12" t="str">
-        <v/>
+        <v>9372281026</v>
       </c>
       <c r="E12" t="str">
         <v/>
       </c>
       <c r="F12" t="str">
+        <v/>
+      </c>
+      <c r="G12" t="str">
+        <v/>
+      </c>
+      <c r="H12" t="str">
+        <v/>
+      </c>
+      <c r="I12" t="str">
+        <v/>
+      </c>
+      <c r="J12" t="str">
+        <v/>
+      </c>
+      <c r="K12" t="str">
+        <v/>
+      </c>
+      <c r="L12" t="str">
+        <v/>
+      </c>
+      <c r="M12" t="str">
+        <v/>
+      </c>
+      <c r="N12" t="str">
+        <v/>
+      </c>
+      <c r="O12" t="str">
+        <v/>
+      </c>
+      <c r="P12" t="str">
+        <v/>
+      </c>
+      <c r="Q12" t="str">
+        <v/>
+      </c>
+      <c r="R12" t="str">
         <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Ayesha Khan</v>
+        <v>AMIT KUMAR</v>
       </c>
       <c r="B13" t="str">
-        <v>C</v>
+        <v>A</v>
       </c>
       <c r="C13" t="str">
-        <v>C-304</v>
+        <v>13</v>
       </c>
       <c r="D13" t="str">
-        <v/>
+        <v>9970962853</v>
       </c>
       <c r="E13" t="str">
         <v/>
       </c>
       <c r="F13" t="str">
-        <v/>
+        <v>Tenant</v>
+      </c>
+      <c r="G13" t="str">
+        <v/>
+      </c>
+      <c r="H13" t="str">
+        <v/>
+      </c>
+      <c r="I13" t="str">
+        <v/>
+      </c>
+      <c r="J13" t="str">
+        <v/>
+      </c>
+      <c r="K13" t="str">
+        <v/>
+      </c>
+      <c r="L13" t="str">
+        <v/>
+      </c>
+      <c r="M13" t="str">
+        <v/>
+      </c>
+      <c r="N13" t="str">
+        <v/>
+      </c>
+      <c r="O13" t="str">
+        <v/>
+      </c>
+      <c r="P13" t="str">
+        <v>NARENDRA SANGHVI</v>
+      </c>
+      <c r="Q13" t="str">
+        <v>8999393126</v>
+      </c>
+      <c r="R13" t="str">
+        <v>Dhanya galli</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Gopal Verma</v>
+        <v>Shripad Pandit Deshpande</v>
       </c>
       <c r="B14" t="str">
-        <v>C</v>
+        <v>B</v>
       </c>
       <c r="C14" t="str">
-        <v>C-405</v>
+        <v>B-8</v>
       </c>
       <c r="D14" t="str">
-        <v/>
+        <v>9422427667</v>
       </c>
       <c r="E14" t="str">
         <v/>
       </c>
       <c r="F14" t="str">
+        <v/>
+      </c>
+      <c r="G14" t="str">
+        <v/>
+      </c>
+      <c r="H14" t="str">
+        <v/>
+      </c>
+      <c r="I14" t="str">
+        <v/>
+      </c>
+      <c r="J14" t="str">
+        <v/>
+      </c>
+      <c r="K14" t="str">
+        <v/>
+      </c>
+      <c r="L14" t="str">
+        <v/>
+      </c>
+      <c r="M14" t="str">
+        <v/>
+      </c>
+      <c r="N14" t="str">
+        <v/>
+      </c>
+      <c r="O14" t="str">
+        <v/>
+      </c>
+      <c r="P14" t="str">
+        <v/>
+      </c>
+      <c r="Q14" t="str">
+        <v/>
+      </c>
+      <c r="R14" t="str">
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Lakshmi Subramanian</v>
+        <v>Vishnu Kumar Malu</v>
       </c>
       <c r="B15" t="str">
-        <v>C</v>
+        <v>B</v>
       </c>
       <c r="C15" t="str">
-        <v>C-506</v>
+        <v>B 3</v>
       </c>
       <c r="D15" t="str">
-        <v/>
+        <v>8830301347</v>
       </c>
       <c r="E15" t="str">
         <v/>
       </c>
       <c r="F15" t="str">
+        <v/>
+      </c>
+      <c r="G15" t="str">
+        <v/>
+      </c>
+      <c r="H15" t="str">
+        <v/>
+      </c>
+      <c r="I15" t="str">
+        <v/>
+      </c>
+      <c r="J15" t="str">
+        <v/>
+      </c>
+      <c r="K15" t="str">
+        <v/>
+      </c>
+      <c r="L15" t="str">
+        <v/>
+      </c>
+      <c r="M15" t="str">
+        <v/>
+      </c>
+      <c r="N15" t="str">
+        <v/>
+      </c>
+      <c r="O15" t="str">
+        <v/>
+      </c>
+      <c r="P15" t="str">
+        <v/>
+      </c>
+      <c r="Q15" t="str">
+        <v/>
+      </c>
+      <c r="R15" t="str">
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Tanvi Mehta</v>
+        <v>Saurabh Khombare</v>
       </c>
       <c r="B16" t="str">
-        <v>C</v>
+        <v>B</v>
       </c>
       <c r="C16" t="str">
-        <v>C-608</v>
+        <v>B-19</v>
       </c>
       <c r="D16" t="str">
-        <v/>
+        <v>9482856848</v>
       </c>
       <c r="E16" t="str">
         <v/>
       </c>
       <c r="F16" t="str">
+        <v/>
+      </c>
+      <c r="G16" t="str">
+        <v/>
+      </c>
+      <c r="H16" t="str">
+        <v/>
+      </c>
+      <c r="I16" t="str">
+        <v/>
+      </c>
+      <c r="J16" t="str">
+        <v/>
+      </c>
+      <c r="K16" t="str">
+        <v/>
+      </c>
+      <c r="L16" t="str">
+        <v/>
+      </c>
+      <c r="M16" t="str">
+        <v/>
+      </c>
+      <c r="N16" t="str">
+        <v/>
+      </c>
+      <c r="O16" t="str">
+        <v/>
+      </c>
+      <c r="P16" t="str">
+        <v/>
+      </c>
+      <c r="Q16" t="str">
+        <v/>
+      </c>
+      <c r="R16" t="str">
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Narendrakumar heda</v>
+        <v>Omnarayan Pannalal jaju</v>
       </c>
       <c r="B17" t="str">
         <v>B</v>
       </c>
       <c r="C17" t="str">
-        <v>11</v>
+        <v>B-7</v>
       </c>
       <c r="D17" t="str">
-        <v>8793109590</v>
+        <v>9423815210</v>
       </c>
       <c r="E17" t="str">
-        <v/>
+        <v>jajuop1960@gmail.com</v>
       </c>
       <c r="F17" t="str">
+        <v/>
+      </c>
+      <c r="G17" t="str">
+        <v/>
+      </c>
+      <c r="H17" t="str">
+        <v/>
+      </c>
+      <c r="I17" t="str">
+        <v/>
+      </c>
+      <c r="J17" t="str">
+        <v/>
+      </c>
+      <c r="K17" t="str">
+        <v/>
+      </c>
+      <c r="L17" t="str">
+        <v/>
+      </c>
+      <c r="M17" t="str">
+        <v/>
+      </c>
+      <c r="N17" t="str">
+        <v/>
+      </c>
+      <c r="O17" t="str">
+        <v/>
+      </c>
+      <c r="P17" t="str">
+        <v/>
+      </c>
+      <c r="Q17" t="str">
+        <v/>
+      </c>
+      <c r="R17" t="str">
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Bhavesh Rajeshkumar Sarda</v>
+        <v>Abhijeet Uday Altekar</v>
       </c>
       <c r="B18" t="str">
-        <v>B</v>
+        <v>A</v>
       </c>
       <c r="C18" t="str">
-        <v>B-2</v>
+        <v>A-17</v>
       </c>
       <c r="D18" t="str">
-        <v>8482996010</v>
+        <v>8698117111</v>
       </c>
       <c r="E18" t="str">
-        <v>bhaveshsarda2004@gmail.com</v>
+        <v>abhijeet.altekar@gmail.com</v>
       </c>
       <c r="F18" t="str">
+        <v/>
+      </c>
+      <c r="G18" t="str">
+        <v/>
+      </c>
+      <c r="H18" t="str">
+        <v/>
+      </c>
+      <c r="I18" t="str">
+        <v/>
+      </c>
+      <c r="J18" t="str">
+        <v/>
+      </c>
+      <c r="K18" t="str">
+        <v/>
+      </c>
+      <c r="L18" t="str">
+        <v/>
+      </c>
+      <c r="M18" t="str">
+        <v/>
+      </c>
+      <c r="N18" t="str">
+        <v/>
+      </c>
+      <c r="O18" t="str">
+        <v/>
+      </c>
+      <c r="P18" t="str">
+        <v/>
+      </c>
+      <c r="Q18" t="str">
+        <v/>
+      </c>
+      <c r="R18" t="str">
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Sagar Agarwal</v>
+        <v>Anil Akiwate</v>
       </c>
       <c r="B19" t="str">
-        <v>A</v>
+        <v>C</v>
       </c>
       <c r="C19" t="str">
-        <v>A - 2</v>
+        <v>C-12</v>
       </c>
       <c r="D19" t="str">
-        <v>7350665037</v>
+        <v>8379805687</v>
       </c>
       <c r="E19" t="str">
-        <v>agarwalsagar016@gmail.com</v>
+        <v>anilakiwate@gmail.com</v>
       </c>
       <c r="F19" t="str">
+        <v/>
+      </c>
+      <c r="G19" t="str">
+        <v/>
+      </c>
+      <c r="H19" t="str">
+        <v/>
+      </c>
+      <c r="I19" t="str">
+        <v/>
+      </c>
+      <c r="J19" t="str">
+        <v/>
+      </c>
+      <c r="K19" t="str">
+        <v/>
+      </c>
+      <c r="L19" t="str">
+        <v/>
+      </c>
+      <c r="M19" t="str">
+        <v/>
+      </c>
+      <c r="N19" t="str">
+        <v/>
+      </c>
+      <c r="O19" t="str">
+        <v/>
+      </c>
+      <c r="P19" t="str">
+        <v/>
+      </c>
+      <c r="Q19" t="str">
+        <v/>
+      </c>
+      <c r="R19" t="str">
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Rahul Pareek</v>
+        <v>Nilesh Koshti</v>
       </c>
       <c r="B20" t="str">
-        <v>B</v>
+        <v>D</v>
       </c>
       <c r="C20" t="str">
-        <v>9</v>
+        <v>D-6</v>
       </c>
       <c r="D20" t="str">
-        <v>9156704040</v>
+        <v>8600204473</v>
       </c>
       <c r="E20" t="str">
-        <v>rahulpareek3366@gmail.com</v>
+        <v>nilesh2348@gmail.com</v>
       </c>
       <c r="F20" t="str">
+        <v/>
+      </c>
+      <c r="G20" t="str">
+        <v/>
+      </c>
+      <c r="H20" t="str">
+        <v/>
+      </c>
+      <c r="I20" t="str">
+        <v/>
+      </c>
+      <c r="J20" t="str">
+        <v/>
+      </c>
+      <c r="K20" t="str">
+        <v/>
+      </c>
+      <c r="L20" t="str">
+        <v/>
+      </c>
+      <c r="M20" t="str">
+        <v/>
+      </c>
+      <c r="N20" t="str">
+        <v/>
+      </c>
+      <c r="O20" t="str">
+        <v/>
+      </c>
+      <c r="P20" t="str">
+        <v/>
+      </c>
+      <c r="Q20" t="str">
+        <v/>
+      </c>
+      <c r="R20" t="str">
         <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Shrihari Narayan Makote</v>
+        <v>Madhavnarayan Rathi</v>
       </c>
       <c r="B21" t="str">
-        <v>D</v>
+        <v>B</v>
       </c>
       <c r="C21" t="str">
-        <v>12</v>
+        <v>B-4</v>
       </c>
       <c r="D21" t="str">
-        <v>9922497427</v>
+        <v>8830149385</v>
       </c>
       <c r="E21" t="str">
-        <v>shriharimakote70@gmail.com</v>
+        <v>mrathi44@gmail.com</v>
       </c>
       <c r="F21" t="str">
         <v/>
       </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="str">
-        <v>Ramdev Rathi</v>
-      </c>
-      <c r="B22" t="str">
-        <v>C</v>
-      </c>
-      <c r="C22" t="str">
-        <v>C2-C3</v>
-      </c>
-      <c r="D22" t="str">
-        <v>9422423985</v>
-      </c>
-      <c r="E22" t="str">
-        <v/>
-      </c>
-      <c r="F22" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="str">
-        <v>Pradeep Jhunjhunwala</v>
-      </c>
-      <c r="B23" t="str">
-        <v>A</v>
-      </c>
-      <c r="C23" t="str">
-        <v>A-10</v>
-      </c>
-      <c r="D23" t="str">
-        <v>9922114900</v>
-      </c>
-      <c r="E23" t="str">
-        <v>cool16yash@gmail.com</v>
-      </c>
-      <c r="F23" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="str">
-        <v>Harishkumar Bharatkumar</v>
-      </c>
-      <c r="B24" t="str">
-        <v>C</v>
-      </c>
-      <c r="C24" t="str">
-        <v>C-14</v>
-      </c>
-      <c r="D24" t="str">
-        <v>7019426263</v>
-      </c>
-      <c r="E24" t="str">
-        <v/>
-      </c>
-      <c r="F24" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="str">
-        <v>Laxmi kant balkrishan malpani</v>
-      </c>
-      <c r="B25" t="str">
-        <v>A</v>
-      </c>
-      <c r="C25" t="str">
-        <v>A/1</v>
-      </c>
-      <c r="D25" t="str">
-        <v>9372281026</v>
-      </c>
-      <c r="E25" t="str">
-        <v/>
-      </c>
-      <c r="F25" t="str">
+      <c r="G21" t="str">
+        <v/>
+      </c>
+      <c r="H21" t="str">
+        <v/>
+      </c>
+      <c r="I21" t="str">
+        <v/>
+      </c>
+      <c r="J21" t="str">
+        <v/>
+      </c>
+      <c r="K21" t="str">
+        <v/>
+      </c>
+      <c r="L21" t="str">
+        <v/>
+      </c>
+      <c r="M21" t="str">
+        <v/>
+      </c>
+      <c r="N21" t="str">
+        <v/>
+      </c>
+      <c r="O21" t="str">
+        <v/>
+      </c>
+      <c r="P21" t="str">
+        <v/>
+      </c>
+      <c r="Q21" t="str">
+        <v/>
+      </c>
+      <c r="R21" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F25"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:R21"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E2"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1649,75 +2398,24 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Society Bye-Laws (2024 revision)</v>
+        <v>Society Bye-Laws</v>
       </c>
       <c r="B2" t="str">
         <v>Governance</v>
       </c>
       <c r="C2" t="str">
-        <v>materials/Society_Bye_Laws_2024.pdf</v>
+        <v>materials/Society_Bye_Laws.pdf</v>
       </c>
       <c r="D2" t="str">
-        <v>2024-06-18</v>
+        <v>2026-01-01</v>
       </c>
       <c r="E2" t="str">
-        <v>Registered bye-laws currently in force</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>AGM Minutes 2025</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Governance</v>
-      </c>
-      <c r="C3" t="str">
-        <v>materials/AGM_Minutes_2025.pdf</v>
-      </c>
-      <c r="D3" t="str">
-        <v>2025-09-20</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Annual general meeting, 14 September 2025</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Maintenance &amp; Water Circular</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Circulars</v>
-      </c>
-      <c r="C4" t="str">
-        <v>materials/Maintenance_Circular_Aug_2025.pdf</v>
-      </c>
-      <c r="D4" t="str">
-        <v>2025-08-01</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Payment dates and revised water timings</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Flat Transfer Application Form</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Forms</v>
-      </c>
-      <c r="C5" t="str">
-        <v>materials/Flat_Transfer_Form.pdf</v>
-      </c>
-      <c r="D5" t="str">
-        <v>2024-11-02</v>
-      </c>
-      <c r="E5" t="str">
-        <v>Submit to the society office with enclosures</v>
+        <v>Upload the file in the admin panel; it fills this row for you</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1891,4 +2589,317 @@
     <ignoredError numberStoredAsText="1" sqref="A1:D11"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:H3"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="17.83203125" customWidth="1"/>
+    <col min="6" max="6" width="20.83203125" customWidth="1"/>
+    <col min="7" max="7" width="14.83203125" customWidth="1"/>
+    <col min="8" max="8" width="23.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Flat</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Person</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Relation</v>
+      </c>
+      <c r="D1" t="str">
+        <v>DOB</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Medical Notes</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Elderly or alone</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Lease Ends</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Police Verification</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>A-101</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Example Owner</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Primary</v>
+      </c>
+      <c r="D2" t="str">
+        <v>1979-04-12</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Diabetic</v>
+      </c>
+      <c r="F2" t="str">
+        <v>No</v>
+      </c>
+      <c r="G2" t="str">
+        <v/>
+      </c>
+      <c r="H2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>B-403</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Example Tenant</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Primary</v>
+      </c>
+      <c r="D3" t="str">
+        <v>1990-08-30</v>
+      </c>
+      <c r="E3" t="str">
+        <v/>
+      </c>
+      <c r="F3" t="str">
+        <v>No</v>
+      </c>
+      <c r="G3" t="str">
+        <v>2027-03-31</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Done 2026-02-10</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:H3"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C18"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Topic</v>
+      </c>
+      <c r="B1" t="str">
+        <v>English</v>
+      </c>
+      <c r="C1" t="str">
+        <v>हिंदी</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Sheets</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Every sheet tab becomes a section on the website, in this order. Add a tab, get a section.</v>
+      </c>
+      <c r="C2" t="str">
+        <v>हर शीट वेबसाइट पर एक अनुभाग बन जाती है। नई शीट जोड़ें, नया अनुभाग बनेगा।</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>About</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Not a section — it fills the page header and holds the settings below.</v>
+      </c>
+      <c r="C3" t="str">
+        <v>यह अनुभाग नहीं है — इससे पेज का शीर्षक और सेटिंग्स बनती हैं।</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Emergency</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Any tab whose name contains "emerg" shows in red in the sidebar.</v>
+      </c>
+      <c r="C4" t="str">
+        <v>जिस शीट के नाम में "emerg" हो, वह साइडबार में लाल रंग में दिखेगी।</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Documents</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Any tab with a File column becomes the documents panel.</v>
+      </c>
+      <c r="C5" t="str">
+        <v>जिस शीट में File कॉलम हो, वह दस्तावेज़ पैनल बन जाएगी।</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Private data</v>
+      </c>
+      <c r="B6" t="str">
+        <v>A sheet or column starting with _ is stored but never shown on the site. Use it for dates of birth.</v>
+      </c>
+      <c r="C6" t="str">
+        <v>_ से शुरू होने वाली शीट या कॉलम वेबसाइट पर कभी नहीं दिखेंगे। जन्मतिथि आदि के लिए इसका उपयोग करें।</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Name column</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Name, Service, Person or Title becomes the card heading.</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Name, Service, Person या Title कार्ड का शीर्षक बनता है।</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Phone column</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Phone, Mobile, Contact No or Cell becomes a call button.</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Phone, Mobile, Contact No या Cell कॉल बटन बन जाता है।</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Role column</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Role, Designation, Post or Type shows as the small label.</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Role, Designation, Post या Type छोटे लेबल के रूप में दिखता है।</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Charges column</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Charges, Rate, Fee or Price shows as a gold badge.</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Charges, Rate, Fee या Price सुनहरे बैज में दिखता है।</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Owner columns</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Owner Name / Owner Phone / Owner Address show behind an "Owner details" button, for tenanted flats.</v>
+      </c>
+      <c r="C11" t="str">
+        <v>किरायेदार वाले फ्लैट के लिए मकान मालिक का विवरण एक बटन के पीछे दिखता है।</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Phone format</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Format phone columns as TEXT in Excel, or it will drop the + and leading zeros.</v>
+      </c>
+      <c r="C12" t="str">
+        <v>फ़ोन कॉलम को Excel में TEXT फ़ॉर्मैट रखें, वरना + और शुरुआती शून्य हट जाएँगे।</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Hindi</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Add "Hindi: &lt;sheet name&gt;" rows in About to translate section names. Values you type are shown as-is, so Hindi names work anywhere.</v>
+      </c>
+      <c r="C13" t="str">
+        <v>अनुभागों के हिंदी नाम About शीट में "Hindi: &lt;नाम&gt;" पंक्ति से जोड़ें। आपके लिखे मान जैसे हैं वैसे दिखते हैं।</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Blood group</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Shown as a red badge on the card. Use a dropdown in your form so you do not collect "o positive" and "O +ve".</v>
+      </c>
+      <c r="C14" t="str">
+        <v>कार्ड पर लाल बैज में दिखता है। फ़ॉर्म में ड्रॉपडाउन रखें।</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Optional fields</v>
+      </c>
+      <c r="B15" t="str">
+        <v>The first two extra columns show on the card; the rest fold behind a More details button. Search still finds them and opens the card.</v>
+      </c>
+      <c r="C15" t="str">
+        <v>पहले दो अतिरिक्त कॉलम कार्ड पर दिखते हैं, बाक़ी "More details" के पीछे। खोज उन्हें भी ढूँढ लेती है।</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>Owner columns</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Fill Owner Name / Owner Phone / Owner Address only for tenanted flats. They appear behind an Owner details button; leave blank and nothing is shown.</v>
+      </c>
+      <c r="C16" t="str">
+        <v>किरायेदार वाले फ्लैट के लिए ही भरें। खाली छोड़ने पर कुछ नहीं दिखेगा।</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>_Private sheet</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Dates of birth, medical notes, lease dates and police verification live here. The leading underscore keeps the sheet off the website entirely.</v>
+      </c>
+      <c r="C17" t="str">
+        <v>जन्मतिथि, चिकित्सा जानकारी आदि यहाँ रखें। यह शीट वेबसाइट पर कभी नहीं दिखती।</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Examples</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Delete the example rows before publishing.</v>
+      </c>
+      <c r="C18" t="str">
+        <v>प्रकाशित करने से पहले उदाहरण पंक्तियाँ हटा दें।</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:C18"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Remove the leftover Services sheet
It duplicated Services & Help as a second, overlapping list on the page.
All ten rows held only a service name — no contact, phone or notes — and
each one already exists as a Role in Services & Help, so nothing is lost.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -9,9 +9,8 @@
     <sheet name="Services &amp; Help" sheetId="4" r:id="rId4"/>
     <sheet name="Residents" sheetId="5" r:id="rId5"/>
     <sheet name="Documents" sheetId="6" r:id="rId6"/>
-    <sheet name="Services" sheetId="7" r:id="rId7"/>
-    <sheet name="_Private" sheetId="8" r:id="rId8"/>
-    <sheet name="_Read me" sheetId="9" r:id="rId9"/>
+    <sheet name="_Private" sheetId="7" r:id="rId7"/>
+    <sheet name="_Read me" sheetId="8" r:id="rId8"/>
   </sheets>
 </workbook>
 </file>
@@ -406,11 +405,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C17"/>
-  <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="34.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -609,13 +603,6 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E3"/>
-  <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="12.83203125" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -678,12 +665,6 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D5"/>
-  <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="12.83203125" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -765,14 +746,6 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F19"/>
-  <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="12.83203125" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" customWidth="1"/>
-    <col min="6" max="6" width="12.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1164,26 +1137,6 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:R21"/>
-  <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="12.83203125" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" customWidth="1"/>
-    <col min="6" max="6" width="12.83203125" customWidth="1"/>
-    <col min="7" max="7" width="15.83203125" customWidth="1"/>
-    <col min="8" max="8" width="21.83203125" customWidth="1"/>
-    <col min="9" max="9" width="14.83203125" customWidth="1"/>
-    <col min="10" max="10" width="16.83203125" customWidth="1"/>
-    <col min="11" max="11" width="16.83203125" customWidth="1"/>
-    <col min="12" max="12" width="14.83203125" customWidth="1"/>
-    <col min="13" max="13" width="12.83203125" customWidth="1"/>
-    <col min="14" max="14" width="13.83203125" customWidth="1"/>
-    <col min="15" max="15" width="12.83203125" customWidth="1"/>
-    <col min="16" max="16" width="14.83203125" customWidth="1"/>
-    <col min="17" max="17" width="15.83203125" customWidth="1"/>
-    <col min="18" max="18" width="17.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2371,13 +2324,6 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E2"/>
-  <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="12.83203125" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2422,188 +2368,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D11"/>
-  <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="12.83203125" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Service</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Contact</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Phone</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Notes</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Plumber</v>
-      </c>
-      <c r="B2" t="str">
-        <v/>
-      </c>
-      <c r="C2" t="str">
-        <v/>
-      </c>
-      <c r="D2" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Electrician</v>
-      </c>
-      <c r="B3" t="str">
-        <v/>
-      </c>
-      <c r="C3" t="str">
-        <v/>
-      </c>
-      <c r="D3" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Lift Technician</v>
-      </c>
-      <c r="B4" t="str">
-        <v/>
-      </c>
-      <c r="C4" t="str">
-        <v/>
-      </c>
-      <c r="D4" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Pest Control</v>
-      </c>
-      <c r="B5" t="str">
-        <v/>
-      </c>
-      <c r="C5" t="str">
-        <v/>
-      </c>
-      <c r="D5" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>Housekeeping</v>
-      </c>
-      <c r="B6" t="str">
-        <v/>
-      </c>
-      <c r="C6" t="str">
-        <v/>
-      </c>
-      <c r="D6" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>Water Tanker</v>
-      </c>
-      <c r="B7" t="str">
-        <v/>
-      </c>
-      <c r="C7" t="str">
-        <v/>
-      </c>
-      <c r="D7" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>Electricity Board</v>
-      </c>
-      <c r="B8" t="str">
-        <v/>
-      </c>
-      <c r="C8" t="str">
-        <v/>
-      </c>
-      <c r="D8" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>Gas Agency</v>
-      </c>
-      <c r="B9" t="str">
-        <v/>
-      </c>
-      <c r="C9" t="str">
-        <v/>
-      </c>
-      <c r="D9" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>Society Manager</v>
-      </c>
-      <c r="B10" t="str">
-        <v/>
-      </c>
-      <c r="C10" t="str">
-        <v/>
-      </c>
-      <c r="D10" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>Accountant</v>
-      </c>
-      <c r="B11" t="str">
-        <v/>
-      </c>
-      <c r="C11" t="str">
-        <v/>
-      </c>
-      <c r="D11" t="str">
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D11"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H3"/>
-  <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="12.83203125" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" customWidth="1"/>
-    <col min="5" max="5" width="17.83203125" customWidth="1"/>
-    <col min="6" max="6" width="20.83203125" customWidth="1"/>
-    <col min="7" max="7" width="14.83203125" customWidth="1"/>
-    <col min="8" max="8" width="23.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2690,14 +2455,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C18"/>
-  <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="12.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">

</xml_diff>

<commit_message>
Drop the members-only banner and keep documents shut until asked for
The banner came from Confidential Notice rows in the About sheet; those
are removed, so nothing renders above the sections. The mechanism stays
for anyone who wants it.

The documents panel now opens on demand. Its heading and file count stay
visible, the list does not — documents are the least urgent thing on the
page and were taking the most room in the sidebar. The choice is
remembered per device, and the heading is keyboard reachable.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -404,7 +404,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C15"/>
+  <cols>
+    <col min="1" max="1" width="26.83203125" customWidth="1"/>
+    <col min="2" max="2" width="80.83203125" customWidth="1"/>
+    <col min="3" max="3" width="46.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -496,43 +501,43 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Confidential Notice</v>
+        <v>Theme</v>
       </c>
       <c r="B9" t="str">
-        <v>Please do not forward this link or share these details with anyone outside the society.</v>
+        <v>Paper</v>
       </c>
       <c r="C9" t="str">
-        <v>ऊपर दिखने वाली चेतावनी (अंग्रेज़ी)</v>
+        <v>navy, forest, plum, slate, sunset, ocean, paper</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Confidential HI</v>
+        <v>Hindi: Committee</v>
       </c>
       <c r="B10" t="str">
-        <v>कृपया यह लिंक या विवरण सोसाइटी के बाहर किसी के साथ साझा न करें।</v>
+        <v>समिति</v>
       </c>
       <c r="C10" t="str">
-        <v>वही चेतावनी हिंदी में</v>
+        <v>हिंदी में अनुभाग का नाम</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Theme</v>
+        <v>Hindi: Emergency</v>
       </c>
       <c r="B11" t="str">
-        <v>Paper</v>
+        <v>आपातकालीन संपर्क</v>
       </c>
       <c r="C11" t="str">
-        <v>navy, forest, plum, slate, sunset, ocean, paper</v>
+        <v>हिंदी में अनुभाग का नाम</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Hindi: Committee</v>
+        <v>Hindi: Services &amp; Help</v>
       </c>
       <c r="B12" t="str">
-        <v>समिति</v>
+        <v>सेवाएँ और सहायता</v>
       </c>
       <c r="C12" t="str">
         <v>हिंदी में अनुभाग का नाम</v>
@@ -540,10 +545,10 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Hindi: Emergency</v>
+        <v>Hindi: Residents</v>
       </c>
       <c r="B13" t="str">
-        <v>आपातकालीन संपर्क</v>
+        <v>निवासी</v>
       </c>
       <c r="C13" t="str">
         <v>हिंदी में अनुभाग का नाम</v>
@@ -551,10 +556,10 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Hindi: Services &amp; Help</v>
+        <v>Hindi: Documents</v>
       </c>
       <c r="B14" t="str">
-        <v>सेवाएँ और सहायता</v>
+        <v>दस्तावेज़</v>
       </c>
       <c r="C14" t="str">
         <v>हिंदी में अनुभाग का नाम</v>
@@ -562,40 +567,18 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Hindi: Residents</v>
+        <v>Note: Services &amp; Help</v>
       </c>
       <c r="B15" t="str">
-        <v>निवासी</v>
+        <v>These contacts are collected from members. They have not been verified or endorsed. Please check credentials and agree charges before engaging anyone — you do so at your own risk.</v>
       </c>
       <c r="C15" t="str">
-        <v>हिंदी में अनुभाग का नाम</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="str">
-        <v>Hindi: Documents</v>
-      </c>
-      <c r="B16" t="str">
-        <v>दस्तावेज़</v>
-      </c>
-      <c r="C16" t="str">
-        <v>हिंदी में अनुभाग का नाम</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="str">
-        <v>Note: Services &amp; Help</v>
-      </c>
-      <c r="B17" t="str">
-        <v>These contacts are collected from members. They have not been verified or endorsed. Please check credentials and agree charges before engaging anyone — you do so at your own risk.</v>
-      </c>
-      <c r="C17" t="str">
         <v>उस अनुभाग के नीचे दिखने वाली चेतावनी</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C17"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C15"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update directory data (78 rows)
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -406,9 +406,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C15"/>
   <cols>
-    <col min="1" max="1" width="26.83203125" customWidth="1"/>
-    <col min="2" max="2" width="80.83203125" customWidth="1"/>
-    <col min="3" max="3" width="46.83203125" customWidth="1"/>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="34.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -586,6 +586,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E3"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -648,6 +655,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D5"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -729,6 +742,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F19"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="12.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -752,42 +773,42 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Santosh Gupta</v>
+        <v>Rahul Shelar</v>
       </c>
       <c r="B2" t="str">
         <v>Plumber</v>
       </c>
       <c r="C2" t="str">
-        <v>₹100 / visit</v>
+        <v/>
       </c>
       <c r="D2" t="str">
         <v>8 AM – 8 PM, on call</v>
       </c>
       <c r="E2" t="str">
-        <v/>
+        <v>9673020210</v>
       </c>
       <c r="F2" t="str">
-        <v>Parts charged separately</v>
+        <v>Plumbing solutions</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Naresh Bhoir</v>
+        <v>Ankush Mhetar</v>
       </c>
       <c r="B3" t="str">
         <v>Electrician</v>
       </c>
       <c r="C3" t="str">
-        <v>₹120 / visit</v>
+        <v/>
       </c>
       <c r="D3" t="str">
         <v>9 AM – 8 PM, on call</v>
       </c>
       <c r="E3" t="str">
-        <v/>
+        <v>9309564191</v>
       </c>
       <c r="F3" t="str">
-        <v>Wiring, fans, MCB</v>
+        <v>Major and Minor electric works</v>
       </c>
     </row>
     <row r="4">
@@ -1120,6 +1141,26 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:R21"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="12.83203125" customWidth="1"/>
+    <col min="7" max="7" width="15.83203125" customWidth="1"/>
+    <col min="8" max="8" width="21.83203125" customWidth="1"/>
+    <col min="9" max="9" width="14.83203125" customWidth="1"/>
+    <col min="10" max="10" width="16.83203125" customWidth="1"/>
+    <col min="11" max="11" width="16.83203125" customWidth="1"/>
+    <col min="12" max="12" width="14.83203125" customWidth="1"/>
+    <col min="13" max="13" width="12.83203125" customWidth="1"/>
+    <col min="14" max="14" width="13.83203125" customWidth="1"/>
+    <col min="15" max="15" width="12.83203125" customWidth="1"/>
+    <col min="16" max="16" width="14.83203125" customWidth="1"/>
+    <col min="17" max="17" width="15.83203125" customWidth="1"/>
+    <col min="18" max="18" width="17.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2307,6 +2348,13 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E2"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2352,6 +2400,16 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H3"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="17.83203125" customWidth="1"/>
+    <col min="6" max="6" width="20.83203125" customWidth="1"/>
+    <col min="7" max="7" width="14.83203125" customWidth="1"/>
+    <col min="8" max="8" width="23.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2441,6 +2499,11 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C18"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">

</xml_diff>

<commit_message>
Update directory data (127 rows)
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -408,6 +408,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F4"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="12.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -500,6 +508,12 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D17"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -749,6 +763,15 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G2"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="12.83203125" customWidth="1"/>
+    <col min="7" max="7" width="12.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -806,6 +829,11 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C19"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="34.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1026,6 +1054,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E3"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1088,6 +1123,12 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D5"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1168,7 +1209,16 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G40"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="12.83203125" customWidth="1"/>
+    <col min="7" max="7" width="12.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1241,148 +1291,148 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Jangid</v>
+        <v>Vaibhav Pest Control</v>
       </c>
       <c r="B4" t="str">
-        <v>Carpenter</v>
+        <v>Pest Control</v>
       </c>
       <c r="C4" t="str">
-        <v>Repairs &amp; Maintenance</v>
+        <v>Building Services</v>
       </c>
       <c r="D4" t="str">
-        <v>₹150 / visit</v>
+        <v/>
       </c>
       <c r="E4" t="str">
-        <v>On call</v>
+        <v/>
       </c>
       <c r="F4" t="str">
-        <v/>
+        <v>9922690290</v>
       </c>
       <c r="G4" t="str">
-        <v>Furniture repair and fittings</v>
+        <v>Quarterly society drive is free</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Otis Service</v>
+        <v/>
       </c>
       <c r="B5" t="str">
-        <v>Lift Technician</v>
+        <v>Gardener</v>
       </c>
       <c r="C5" t="str">
         <v>Building Services</v>
       </c>
       <c r="D5" t="str">
-        <v>Society AMC</v>
+        <v/>
       </c>
       <c r="E5" t="str">
-        <v>4-hour response</v>
+        <v/>
       </c>
       <c r="F5" t="str">
         <v/>
       </c>
       <c r="G5" t="str">
-        <v>Report faults to the manager first</v>
+        <v>Balcony and terrace plants</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>HiCare</v>
+        <v/>
       </c>
       <c r="B6" t="str">
-        <v>Pest Control</v>
+        <v>Gas Agency</v>
       </c>
       <c r="C6" t="str">
-        <v>Building Services</v>
+        <v>Utilities</v>
       </c>
       <c r="D6" t="str">
-        <v>₹1,200 / flat</v>
+        <v/>
       </c>
       <c r="E6" t="str">
-        <v>By appointment</v>
+        <v/>
       </c>
       <c r="F6" t="str">
         <v/>
       </c>
       <c r="G6" t="str">
-        <v>Quarterly society drive is free</v>
+        <v>Leak helpline 1800 22 9944</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Shanti Devi</v>
+        <v>Akka Maushi</v>
       </c>
       <c r="B7" t="str">
-        <v>Housekeeping</v>
+        <v>Maid</v>
       </c>
       <c r="C7" t="str">
-        <v>Building Services</v>
+        <v>Home Help</v>
       </c>
       <c r="D7" t="str">
-        <v>Society staff</v>
+        <v/>
       </c>
       <c r="E7" t="str">
-        <v>6 AM – 2 PM</v>
+        <v/>
       </c>
       <c r="F7" t="str">
-        <v/>
+        <v>9922090766</v>
       </c>
       <c r="G7" t="str">
-        <v>Common areas and staircases</v>
+        <v>Sweeping, mopping, utensils</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Ganesh Pawar</v>
+        <v>Sunita Maushi</v>
       </c>
       <c r="B8" t="str">
-        <v>Gardener</v>
+        <v>Maid</v>
       </c>
       <c r="C8" t="str">
-        <v>Building Services</v>
+        <v>Home Help</v>
       </c>
       <c r="D8" t="str">
-        <v>₹80 / visit</v>
+        <v/>
       </c>
       <c r="E8" t="str">
-        <v>Tue &amp; Sat mornings</v>
+        <v/>
       </c>
       <c r="F8" t="str">
-        <v/>
+        <v>7249544168</v>
       </c>
       <c r="G8" t="str">
-        <v>Balcony and terrace plants</v>
+        <v>Sweeping, mopping, utensils</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Jai Bhavani</v>
+        <v/>
       </c>
       <c r="B9" t="str">
-        <v>Water Tanker</v>
+        <v>Driver</v>
       </c>
       <c r="C9" t="str">
-        <v>Utilities</v>
+        <v>Home Help</v>
       </c>
       <c r="D9" t="str">
-        <v>₹900 / tanker</v>
+        <v/>
       </c>
       <c r="E9" t="str">
-        <v>Same-day delivery</v>
+        <v/>
       </c>
       <c r="F9" t="str">
         <v/>
       </c>
       <c r="G9" t="str">
-        <v>10,000 litre tanker</v>
+        <v>Local trips, holds a valid licence</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>MSEDCL</v>
+        <v>aditya wireman</v>
       </c>
       <c r="B10" t="str">
-        <v>Electricity Board</v>
+        <v>Electrician</v>
       </c>
       <c r="C10" t="str">
         <v>Utilities</v>
@@ -1391,21 +1441,21 @@
         <v/>
       </c>
       <c r="E10" t="str">
-        <v>24x7 helpline</v>
+        <v/>
       </c>
       <c r="F10" t="str">
-        <v/>
+        <v>9325680187</v>
       </c>
       <c r="G10" t="str">
-        <v>Outages and meter faults</v>
+        <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Mahanagar Gas</v>
+        <v>Awade mseb</v>
       </c>
       <c r="B11" t="str">
-        <v>Gas Agency</v>
+        <v>Electricity Board</v>
       </c>
       <c r="C11" t="str">
         <v>Utilities</v>
@@ -1414,202 +1464,685 @@
         <v/>
       </c>
       <c r="E11" t="str">
-        <v>24x7 for leaks</v>
+        <v/>
       </c>
       <c r="F11" t="str">
-        <v/>
+        <v>7875936797</v>
       </c>
       <c r="G11" t="str">
-        <v>Leak helpline 1800 22 9944</v>
+        <v>MSEB office awade</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>D. Kamble</v>
+        <v>Ramesh patil Boring</v>
       </c>
       <c r="B12" t="str">
-        <v>Society Manager</v>
+        <v/>
       </c>
       <c r="C12" t="str">
-        <v>Society Staff</v>
+        <v>Utilities</v>
       </c>
       <c r="D12" t="str">
         <v/>
       </c>
       <c r="E12" t="str">
-        <v>Mon–Sat, 10 AM – 6 PM</v>
+        <v/>
       </c>
       <c r="F12" t="str">
-        <v/>
+        <v>9850929761</v>
       </c>
       <c r="G12" t="str">
-        <v>Maintenance bills, NOCs, complaints</v>
+        <v>Boring repair work</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>S. Rane</v>
+        <v>Ramesh patil Boring 1</v>
       </c>
       <c r="B13" t="str">
-        <v>Accountant</v>
+        <v/>
       </c>
       <c r="C13" t="str">
-        <v>Society Staff</v>
+        <v/>
       </c>
       <c r="D13" t="str">
         <v/>
       </c>
       <c r="E13" t="str">
-        <v>Tue &amp; Thu, 4 PM – 7 PM</v>
+        <v/>
       </c>
       <c r="F13" t="str">
-        <v/>
+        <v>9503814294</v>
       </c>
       <c r="G13" t="str">
-        <v>Dues, receipts, statements</v>
+        <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Sunita Bai</v>
+        <v>Vishal Boring Repare</v>
       </c>
       <c r="B14" t="str">
-        <v>Maid</v>
+        <v/>
       </c>
       <c r="C14" t="str">
-        <v>Home Help</v>
+        <v/>
       </c>
       <c r="D14" t="str">
-        <v>₹50 / visit</v>
+        <v/>
       </c>
       <c r="E14" t="str">
-        <v>7 AM – 11 AM</v>
+        <v/>
       </c>
       <c r="F14" t="str">
-        <v/>
+        <v>9028650650</v>
       </c>
       <c r="G14" t="str">
-        <v>Sweeping, mopping, utensils</v>
+        <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Lata Devi</v>
+        <v>Vinyak Boring Senser</v>
       </c>
       <c r="B15" t="str">
-        <v>Maid</v>
+        <v/>
       </c>
       <c r="C15" t="str">
-        <v>Home Help</v>
+        <v/>
       </c>
       <c r="D15" t="str">
-        <v>₹60 / visit</v>
+        <v/>
       </c>
       <c r="E15" t="str">
-        <v>6 AM – 10 AM</v>
+        <v/>
       </c>
       <c r="F15" t="str">
-        <v/>
+        <v>9168921005</v>
       </c>
       <c r="G15" t="str">
-        <v>Also irons clothes on request</v>
+        <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Kamla Bai</v>
+        <v>Ravi patil Boring Repare</v>
       </c>
       <c r="B16" t="str">
-        <v>Cook</v>
+        <v/>
       </c>
       <c r="C16" t="str">
-        <v>Home Help</v>
+        <v/>
       </c>
       <c r="D16" t="str">
-        <v>₹2,500 / month</v>
+        <v/>
       </c>
       <c r="E16" t="str">
-        <v>11 AM – 2 PM</v>
+        <v/>
       </c>
       <c r="F16" t="str">
-        <v/>
+        <v>8788731240</v>
       </c>
       <c r="G16" t="str">
-        <v>Vegetarian, two meals a day</v>
+        <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>ganesh raju</v>
+        <v>Shrinivsh Boring</v>
       </c>
       <c r="B17" t="str">
-        <v>Car Cleaning</v>
+        <v/>
       </c>
       <c r="C17" t="str">
-        <v>Home Help</v>
+        <v/>
       </c>
       <c r="D17" t="str">
-        <v>₹500 / month</v>
+        <v/>
       </c>
       <c r="E17" t="str">
-        <v>6 AM – 9 AM</v>
+        <v/>
       </c>
       <c r="F17" t="str">
-        <v/>
+        <v>8855961649</v>
       </c>
       <c r="G17" t="str">
-        <v>Daily wash, interior weekly</v>
+        <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Deepak Sawant</v>
+        <v>Pravin Lavate IMC Clerk</v>
       </c>
       <c r="B18" t="str">
-        <v>Driver</v>
+        <v/>
       </c>
       <c r="C18" t="str">
-        <v>Home Help</v>
+        <v>Utilities</v>
       </c>
       <c r="D18" t="str">
-        <v>₹300 / trip</v>
+        <v/>
       </c>
       <c r="E18" t="str">
-        <v>By appointment</v>
+        <v/>
       </c>
       <c r="F18" t="str">
-        <v/>
+        <v>9922772149</v>
       </c>
       <c r="G18" t="str">
-        <v>Local trips, holds a valid licence</v>
+        <v>Property tax related officer</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Anita Kamble</v>
+        <v>Solanky Madam Sanitary Incepector IMC</v>
       </c>
       <c r="B19" t="str">
-        <v>Baby Sitter</v>
+        <v/>
       </c>
       <c r="C19" t="str">
-        <v>Home Help</v>
+        <v>Utilities</v>
       </c>
       <c r="D19" t="str">
-        <v>₹150 / hour</v>
+        <v/>
       </c>
       <c r="E19" t="str">
-        <v>Flexible</v>
+        <v/>
       </c>
       <c r="F19" t="str">
-        <v/>
+        <v>8329253329</v>
       </c>
       <c r="G19" t="str">
-        <v>Experienced with toddlers</v>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>Ghanta Gadi Ankush Kurne</v>
+      </c>
+      <c r="B20" t="str">
+        <v/>
+      </c>
+      <c r="C20" t="str">
+        <v>Utilities</v>
+      </c>
+      <c r="D20" t="str">
+        <v/>
+      </c>
+      <c r="E20" t="str">
+        <v/>
+      </c>
+      <c r="F20" t="str">
+        <v>9146111279</v>
+      </c>
+      <c r="G20" t="str">
+        <v>Garbage van</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Alliance Hospital Ich</v>
+      </c>
+      <c r="B21" t="str">
+        <v/>
+      </c>
+      <c r="C21" t="str">
+        <v>Hospital</v>
+      </c>
+      <c r="D21" t="str">
+        <v/>
+      </c>
+      <c r="E21" t="str">
+        <v/>
+      </c>
+      <c r="F21" t="str">
+        <v>0230 2435001</v>
+      </c>
+      <c r="G21" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>mseb Wireman Rohit</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Electricity Board</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Utilities</v>
+      </c>
+      <c r="D22" t="str">
+        <v/>
+      </c>
+      <c r="E22" t="str">
+        <v/>
+      </c>
+      <c r="F22" t="str">
+        <v>9762315904</v>
+      </c>
+      <c r="G22" t="str">
+        <v>MSEB Wireman</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>Ich S T Depot</v>
+      </c>
+      <c r="B23" t="str">
+        <v/>
+      </c>
+      <c r="C23" t="str">
+        <v>Utilities</v>
+      </c>
+      <c r="D23" t="str">
+        <v/>
+      </c>
+      <c r="E23" t="str">
+        <v/>
+      </c>
+      <c r="F23" t="str">
+        <v>0230 2432496</v>
+      </c>
+      <c r="G23" t="str">
+        <v xml:space="preserve">Bus depot </v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v xml:space="preserve">Ich S T  Stand </v>
+      </c>
+      <c r="B24" t="str">
+        <v/>
+      </c>
+      <c r="C24" t="str">
+        <v>Utilities</v>
+      </c>
+      <c r="D24" t="str">
+        <v/>
+      </c>
+      <c r="E24" t="str">
+        <v/>
+      </c>
+      <c r="F24" t="str">
+        <v>0230 2432202</v>
+      </c>
+      <c r="G24" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v xml:space="preserve">seva bharti Hospital </v>
+      </c>
+      <c r="B25" t="str">
+        <v/>
+      </c>
+      <c r="C25" t="str">
+        <v>Hospital</v>
+      </c>
+      <c r="D25" t="str">
+        <v/>
+      </c>
+      <c r="E25" t="str">
+        <v/>
+      </c>
+      <c r="F25" t="str">
+        <v>0230 2426171</v>
+      </c>
+      <c r="G25" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>Ich S T Venktesh Parking Stand</v>
+      </c>
+      <c r="B26" t="str">
+        <v/>
+      </c>
+      <c r="C26" t="str">
+        <v>Utilities</v>
+      </c>
+      <c r="D26" t="str">
+        <v/>
+      </c>
+      <c r="E26" t="str">
+        <v/>
+      </c>
+      <c r="F26" t="str">
+        <v>8237744444</v>
+      </c>
+      <c r="G26" t="str">
+        <v>Parking at bus stand</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>S T Ich</v>
+      </c>
+      <c r="B27" t="str">
+        <v/>
+      </c>
+      <c r="C27" t="str">
+        <v>Utilities</v>
+      </c>
+      <c r="D27" t="str">
+        <v/>
+      </c>
+      <c r="E27" t="str">
+        <v/>
+      </c>
+      <c r="F27" t="str">
+        <v>0230 2432202</v>
+      </c>
+      <c r="G27" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>Aadhar Blood Bank Mete Saheb</v>
+      </c>
+      <c r="B28" t="str">
+        <v/>
+      </c>
+      <c r="C28" t="str">
+        <v>Utilities</v>
+      </c>
+      <c r="D28" t="str">
+        <v/>
+      </c>
+      <c r="E28" t="str">
+        <v/>
+      </c>
+      <c r="F28" t="str">
+        <v>8149370204</v>
+      </c>
+      <c r="G28" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>Amrutmama Bhosale</v>
+      </c>
+      <c r="B29" t="str">
+        <v/>
+      </c>
+      <c r="C29" t="str">
+        <v>Nagarsevak</v>
+      </c>
+      <c r="D29" t="str">
+        <v/>
+      </c>
+      <c r="E29" t="str">
+        <v/>
+      </c>
+      <c r="F29" t="str">
+        <v>9975067101</v>
+      </c>
+      <c r="G29" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>Raju Pujari Balaji Bakery</v>
+      </c>
+      <c r="B30" t="str">
+        <v/>
+      </c>
+      <c r="C30" t="str">
+        <v>Nagarsevak</v>
+      </c>
+      <c r="D30" t="str">
+        <v/>
+      </c>
+      <c r="E30" t="str">
+        <v/>
+      </c>
+      <c r="F30" t="str">
+        <v>9021543640</v>
+      </c>
+      <c r="G30" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>Nagesh Patil Dada</v>
+      </c>
+      <c r="B31" t="str">
+        <v/>
+      </c>
+      <c r="C31" t="str">
+        <v>Nagarsevak</v>
+      </c>
+      <c r="D31" t="str">
+        <v/>
+      </c>
+      <c r="E31" t="str">
+        <v/>
+      </c>
+      <c r="F31" t="str">
+        <v>8888341342</v>
+      </c>
+      <c r="G31" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>Nagesh Patil Dada</v>
+      </c>
+      <c r="B32" t="str">
+        <v/>
+      </c>
+      <c r="C32" t="str">
+        <v>Nagarsevak</v>
+      </c>
+      <c r="D32" t="str">
+        <v/>
+      </c>
+      <c r="E32" t="str">
+        <v/>
+      </c>
+      <c r="F32" t="str">
+        <v>8888341342</v>
+      </c>
+      <c r="G32" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>Santosh Shelke</v>
+      </c>
+      <c r="B33" t="str">
+        <v/>
+      </c>
+      <c r="C33" t="str">
+        <v>Nagarsevak</v>
+      </c>
+      <c r="D33" t="str">
+        <v/>
+      </c>
+      <c r="E33" t="str">
+        <v/>
+      </c>
+      <c r="F33" t="str">
+        <v>9423040242</v>
+      </c>
+      <c r="G33" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>LV Gate Watchman Uttam</v>
+      </c>
+      <c r="B34" t="str">
+        <v/>
+      </c>
+      <c r="C34" t="str">
+        <v>Society Staff</v>
+      </c>
+      <c r="D34" t="str">
+        <v/>
+      </c>
+      <c r="E34" t="str">
+        <v/>
+      </c>
+      <c r="F34" t="str">
+        <v>9595405090</v>
+      </c>
+      <c r="G34" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>LV Gate Watchman Umesh Patil</v>
+      </c>
+      <c r="B35" t="str">
+        <v/>
+      </c>
+      <c r="C35" t="str">
+        <v>Society Staff</v>
+      </c>
+      <c r="D35" t="str">
+        <v/>
+      </c>
+      <c r="E35" t="str">
+        <v/>
+      </c>
+      <c r="F35" t="str">
+        <v>9970327078</v>
+      </c>
+      <c r="G35" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>LV Watchman Lokere</v>
+      </c>
+      <c r="B36" t="str">
+        <v/>
+      </c>
+      <c r="C36" t="str">
+        <v>Society Staff</v>
+      </c>
+      <c r="D36" t="str">
+        <v/>
+      </c>
+      <c r="E36" t="str">
+        <v/>
+      </c>
+      <c r="F36" t="str">
+        <v>9075242921</v>
+      </c>
+      <c r="G36" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>L V Lift Shravani Costmer Care</v>
+      </c>
+      <c r="B37" t="str">
+        <v/>
+      </c>
+      <c r="C37" t="str">
+        <v>Society Staff</v>
+      </c>
+      <c r="D37" t="str">
+        <v/>
+      </c>
+      <c r="E37" t="str">
+        <v/>
+      </c>
+      <c r="F37" t="str">
+        <v>7744888217</v>
+      </c>
+      <c r="G37" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>LV Lift Vijay Parker</v>
+      </c>
+      <c r="B38" t="str">
+        <v/>
+      </c>
+      <c r="C38" t="str">
+        <v>Society Staff</v>
+      </c>
+      <c r="D38" t="str">
+        <v/>
+      </c>
+      <c r="E38" t="str">
+        <v/>
+      </c>
+      <c r="F38" t="str">
+        <v>8087508217</v>
+      </c>
+      <c r="G38" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>LV Lift Pradeep</v>
+      </c>
+      <c r="B39" t="str">
+        <v/>
+      </c>
+      <c r="C39" t="str">
+        <v>Society Staff</v>
+      </c>
+      <c r="D39" t="str">
+        <v/>
+      </c>
+      <c r="E39" t="str">
+        <v/>
+      </c>
+      <c r="F39" t="str">
+        <v>9082264006</v>
+      </c>
+      <c r="G39" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>Police Crane Vishal</v>
+      </c>
+      <c r="B40" t="str">
+        <v/>
+      </c>
+      <c r="C40" t="str">
+        <v/>
+      </c>
+      <c r="D40" t="str">
+        <v/>
+      </c>
+      <c r="E40" t="str">
+        <v/>
+      </c>
+      <c r="F40" t="str">
+        <v>8421410046</v>
+      </c>
+      <c r="G40" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G19"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G40"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1617,6 +2150,27 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:S21"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="13.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="12.83203125" customWidth="1"/>
+    <col min="7" max="7" width="12.83203125" customWidth="1"/>
+    <col min="8" max="8" width="15.83203125" customWidth="1"/>
+    <col min="9" max="9" width="21.83203125" customWidth="1"/>
+    <col min="10" max="10" width="14.83203125" customWidth="1"/>
+    <col min="11" max="11" width="16.83203125" customWidth="1"/>
+    <col min="12" max="12" width="16.83203125" customWidth="1"/>
+    <col min="13" max="13" width="14.83203125" customWidth="1"/>
+    <col min="14" max="14" width="12.83203125" customWidth="1"/>
+    <col min="15" max="15" width="13.83203125" customWidth="1"/>
+    <col min="16" max="16" width="12.83203125" customWidth="1"/>
+    <col min="17" max="17" width="14.83203125" customWidth="1"/>
+    <col min="18" max="18" width="15.83203125" customWidth="1"/>
+    <col min="19" max="19" width="17.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2867,6 +3421,13 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E2"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2912,6 +3473,16 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H3"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="17.83203125" customWidth="1"/>
+    <col min="6" max="6" width="20.83203125" customWidth="1"/>
+    <col min="7" max="7" width="14.83203125" customWidth="1"/>
+    <col min="8" max="8" width="23.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3001,6 +3572,11 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C22"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">

</xml_diff>

<commit_message>
Update directory data (134 rows)
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -2149,7 +2149,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S21"/>
+  <dimension ref="A1:S28"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -3411,9 +3411,422 @@
         <v/>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>Radheshyam Narayanlal Loya</v>
+      </c>
+      <c r="B22" t="str">
+        <v>B</v>
+      </c>
+      <c r="C22" t="str">
+        <v>B-5</v>
+      </c>
+      <c r="D22" t="str">
+        <v/>
+      </c>
+      <c r="E22" t="str">
+        <v>9422414549</v>
+      </c>
+      <c r="F22" t="str">
+        <v/>
+      </c>
+      <c r="G22" t="str">
+        <v/>
+      </c>
+      <c r="H22" t="str">
+        <v>O+</v>
+      </c>
+      <c r="I22" t="str">
+        <v/>
+      </c>
+      <c r="J22" t="str">
+        <v/>
+      </c>
+      <c r="K22" t="str">
+        <v/>
+      </c>
+      <c r="L22" t="str">
+        <v/>
+      </c>
+      <c r="M22" t="str">
+        <v/>
+      </c>
+      <c r="N22" t="str">
+        <v/>
+      </c>
+      <c r="O22" t="str">
+        <v/>
+      </c>
+      <c r="P22" t="str">
+        <v/>
+      </c>
+      <c r="Q22" t="str">
+        <v/>
+      </c>
+      <c r="R22" t="str">
+        <v/>
+      </c>
+      <c r="S22" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>prasad kulkarni</v>
+      </c>
+      <c r="B23" t="str">
+        <v>D</v>
+      </c>
+      <c r="C23" t="str">
+        <v>D10</v>
+      </c>
+      <c r="D23" t="str">
+        <v/>
+      </c>
+      <c r="E23" t="str">
+        <v>8483098383</v>
+      </c>
+      <c r="F23" t="str">
+        <v/>
+      </c>
+      <c r="G23" t="str">
+        <v/>
+      </c>
+      <c r="H23" t="str">
+        <v>B +ve</v>
+      </c>
+      <c r="I23" t="str">
+        <v/>
+      </c>
+      <c r="J23" t="str">
+        <v/>
+      </c>
+      <c r="K23" t="str">
+        <v/>
+      </c>
+      <c r="L23" t="str">
+        <v/>
+      </c>
+      <c r="M23" t="str">
+        <v/>
+      </c>
+      <c r="N23" t="str">
+        <v/>
+      </c>
+      <c r="O23" t="str">
+        <v/>
+      </c>
+      <c r="P23" t="str">
+        <v/>
+      </c>
+      <c r="Q23" t="str">
+        <v/>
+      </c>
+      <c r="R23" t="str">
+        <v/>
+      </c>
+      <c r="S23" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>Gourav Pujari</v>
+      </c>
+      <c r="B24" t="str">
+        <v>D</v>
+      </c>
+      <c r="C24" t="str">
+        <v>D-18</v>
+      </c>
+      <c r="D24" t="str">
+        <v/>
+      </c>
+      <c r="E24" t="str">
+        <v>7276440440</v>
+      </c>
+      <c r="F24" t="str">
+        <v/>
+      </c>
+      <c r="G24" t="str">
+        <v/>
+      </c>
+      <c r="H24" t="str">
+        <v>A+</v>
+      </c>
+      <c r="I24" t="str">
+        <v/>
+      </c>
+      <c r="J24" t="str">
+        <v/>
+      </c>
+      <c r="K24" t="str">
+        <v/>
+      </c>
+      <c r="L24" t="str">
+        <v/>
+      </c>
+      <c r="M24" t="str">
+        <v/>
+      </c>
+      <c r="N24" t="str">
+        <v/>
+      </c>
+      <c r="O24" t="str">
+        <v/>
+      </c>
+      <c r="P24" t="str">
+        <v/>
+      </c>
+      <c r="Q24" t="str">
+        <v/>
+      </c>
+      <c r="R24" t="str">
+        <v/>
+      </c>
+      <c r="S24" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>Nilesh Suresh Koshti</v>
+      </c>
+      <c r="B25" t="str">
+        <v>D</v>
+      </c>
+      <c r="C25" t="str">
+        <v>D6</v>
+      </c>
+      <c r="D25" t="str">
+        <v/>
+      </c>
+      <c r="E25" t="str">
+        <v>8600204473</v>
+      </c>
+      <c r="F25" t="str">
+        <v>nilesh2348@gmail.com</v>
+      </c>
+      <c r="G25" t="str">
+        <v/>
+      </c>
+      <c r="H25" t="str">
+        <v>B+</v>
+      </c>
+      <c r="I25" t="str">
+        <v/>
+      </c>
+      <c r="J25" t="str">
+        <v/>
+      </c>
+      <c r="K25" t="str">
+        <v/>
+      </c>
+      <c r="L25" t="str">
+        <v/>
+      </c>
+      <c r="M25" t="str">
+        <v/>
+      </c>
+      <c r="N25" t="str">
+        <v/>
+      </c>
+      <c r="O25" t="str">
+        <v>4</v>
+      </c>
+      <c r="P25" t="str">
+        <v/>
+      </c>
+      <c r="Q25" t="str">
+        <v/>
+      </c>
+      <c r="R25" t="str">
+        <v/>
+      </c>
+      <c r="S25" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>Adv. Omkar Smita Mahaveer Kurade</v>
+      </c>
+      <c r="B26" t="str">
+        <v>A</v>
+      </c>
+      <c r="C26" t="str">
+        <v>A-8</v>
+      </c>
+      <c r="D26" t="str">
+        <v/>
+      </c>
+      <c r="E26" t="str">
+        <v>9762226311</v>
+      </c>
+      <c r="F26" t="str">
+        <v>advomkarkurade@gmail.com</v>
+      </c>
+      <c r="G26" t="str">
+        <v/>
+      </c>
+      <c r="H26" t="str">
+        <v>A+</v>
+      </c>
+      <c r="I26" t="str">
+        <v/>
+      </c>
+      <c r="J26" t="str">
+        <v/>
+      </c>
+      <c r="K26" t="str">
+        <v/>
+      </c>
+      <c r="L26" t="str">
+        <v/>
+      </c>
+      <c r="M26" t="str">
+        <v>Advocate</v>
+      </c>
+      <c r="N26" t="str">
+        <v/>
+      </c>
+      <c r="O26" t="str">
+        <v>4</v>
+      </c>
+      <c r="P26" t="str">
+        <v/>
+      </c>
+      <c r="Q26" t="str">
+        <v/>
+      </c>
+      <c r="R26" t="str">
+        <v/>
+      </c>
+      <c r="S26" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>Shashikant Joshi</v>
+      </c>
+      <c r="B27" t="str">
+        <v>C</v>
+      </c>
+      <c r="C27" t="str">
+        <v>B-12</v>
+      </c>
+      <c r="D27" t="str">
+        <v/>
+      </c>
+      <c r="E27" t="str">
+        <v>9011074074</v>
+      </c>
+      <c r="F27" t="str">
+        <v/>
+      </c>
+      <c r="G27" t="str">
+        <v/>
+      </c>
+      <c r="H27" t="str">
+        <v>B+</v>
+      </c>
+      <c r="I27" t="str">
+        <v/>
+      </c>
+      <c r="J27" t="str">
+        <v/>
+      </c>
+      <c r="K27" t="str">
+        <v/>
+      </c>
+      <c r="L27" t="str">
+        <v/>
+      </c>
+      <c r="M27" t="str">
+        <v/>
+      </c>
+      <c r="N27" t="str">
+        <v/>
+      </c>
+      <c r="O27" t="str">
+        <v>4</v>
+      </c>
+      <c r="P27" t="str">
+        <v/>
+      </c>
+      <c r="Q27" t="str">
+        <v/>
+      </c>
+      <c r="R27" t="str">
+        <v/>
+      </c>
+      <c r="S27" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>Vishal Suresh kolekar</v>
+      </c>
+      <c r="B28" t="str">
+        <v>D</v>
+      </c>
+      <c r="C28" t="str">
+        <v>D 7</v>
+      </c>
+      <c r="D28" t="str">
+        <v/>
+      </c>
+      <c r="E28" t="str">
+        <v>9623880919</v>
+      </c>
+      <c r="F28" t="str">
+        <v/>
+      </c>
+      <c r="G28" t="str">
+        <v/>
+      </c>
+      <c r="H28" t="str">
+        <v>AB+</v>
+      </c>
+      <c r="I28" t="str">
+        <v/>
+      </c>
+      <c r="J28" t="str">
+        <v/>
+      </c>
+      <c r="K28" t="str">
+        <v/>
+      </c>
+      <c r="L28" t="str">
+        <v/>
+      </c>
+      <c r="M28" t="str">
+        <v/>
+      </c>
+      <c r="N28" t="str">
+        <v/>
+      </c>
+      <c r="O28" t="str">
+        <v>3</v>
+      </c>
+      <c r="P28" t="str">
+        <v/>
+      </c>
+      <c r="Q28" t="str">
+        <v/>
+      </c>
+      <c r="R28" t="str">
+        <v/>
+      </c>
+      <c r="S28" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S28"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>